<commit_message>
Step 3c: review batch 01 — Regional Optimization & Refinery Planning
</commit_message>
<xml_diff>
--- a/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
+++ b/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review &amp; authoring'!$A$1:$AD$504</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Controlled vocabularies'!$A$3:$C$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Reference register'!$A$7:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Reference register'!$A$7:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'External mappings'!$A$8:$K$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1752,18 +1752,85 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U11" s="5" t="n"/>
-      <c r="V11" s="5" t="n"/>
-      <c r="W11" s="5" t="n"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Assign available crude and feedstock cargoes, grades, and volumes to specific refineries and receipt windows so each site's approved production plan can be met at the best delivered economics across the region.</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Covers the recurring allocation of secured or available crude and feedstock supply across competing refinery destinations, including grade-to-site matching, volume splits, timing of receipt windows, and reallocation when supply or plan assumptions change. Excludes crude purchase, negotiation, and trade execution, owned by Supply And Trading; excludes vessel, pipeline, and terminal movement execution, owned by Midstream; excludes the refinery's internal decision on which tanks and units process an allocated grade, owned by Refining.</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Grade-to-refinery assignment | volume split across sites | receipt-window timing | reallocation on supply disruption or plan change | allocation of term and spot volumes against planned refinery slates</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Crude purchasing and trade execution (Supply And Trading) | physical movement, berth and pipeline scheduling (Midstream) | unit-level crude processing decisions (Refining) | refinery slate economics selection (Refinery Planning)</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Crude Allocation | Feedstock Allocation | Crude &amp; Feedstock Allocation</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Allocate Term Crude Volumes | Allocate Spot Crude Volumes | Reallocate Crude on Supply Disruption</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Label retains the existing “Decision” suffix, but the concept is authored as the recurring allocation process, not the decision record or its output. A later naming pass should consider “Allocate Crude &amp; Feedstock” for verb consistency with sibling labels; not changed in this batch. The boundary against Supply And Trading follows the locked SCM/Commercial rule: this concept places already-secured supply and does not choose counterparty, price, or contract.</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>Decide which refinery receives which crude and feedstock volumes, and when, so the regional plan is met at best delivered economics.</t>
+        </is>
+      </c>
+      <c r="W11" s="5" t="inlineStr">
+        <is>
+          <t>SRC-CMU-REFPLAN-001 | SRC-SNF-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X11" s="5" t="n"/>
-      <c r="Y11" s="5" t="n"/>
-      <c r="Z11" s="5" t="n"/>
-      <c r="AA11" s="5" t="n"/>
-      <c r="AB11" s="5" t="n"/>
-      <c r="AC11" s="5" t="n"/>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
+          <t>approved refinery production plan | secured and available crude supply position | crude and feedstock quality assays | delivered-cost and freight economics | refinery receipt and storage constraints</t>
+        </is>
+      </c>
+      <c r="Z11" s="5" t="inlineStr">
+        <is>
+          <t>approved crude and feedstock allocation to refineries and receipt windows</t>
+        </is>
+      </c>
+      <c r="AA11" s="5" t="inlineStr">
+        <is>
+          <t>informed-by: Refinery Planning | constrained-by: Inventory | precedes: Refinery Scheduling</t>
+        </is>
+      </c>
+      <c r="AB11" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC11" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1831,18 +1898,85 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U12" s="5" t="n"/>
-      <c r="V12" s="5" t="n"/>
-      <c r="W12" s="5" t="n"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Assign available finished-product supply to markets, channels, terminals, and customer commitments for a planning period, so limited or constrained volumes are placed where they best serve contractual obligations and regional margin.</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Covers plan-level placement of finished product across markets, channels, and supply points, including the commercial priority rules applied when available supply cannot meet all demand, and reallocation when supply, demand, or logistics change. Excludes order-level allocation and release against an individual customer order, owned by Order Management; excludes rack and terminal loading allocation enforcement, owned by Terminal Loading; excludes physical movement and delivery execution, owned by Midstream and Distribution.</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Market and channel volume placement | supply-point-to-demand-point assignment | commercial priority rules under constrained supply | exchange and third-party placement within the plan | reallocation on plan change</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Order-level allocation and release (Allocate &amp; Release Order, Order Management) | rack and terminal allocation enforcement (Manage Allocation, Terminal Loading) | sales-target setting (Determine &amp; Allocate Sales Targets, Marketing) | pricing and offer construction (Commercial &amp; Marketing pricing processes) | physical delivery (Midstream, Distribution)</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Product Allocation | Finished Product Allocation | Supply Allocation</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Define Product Allocation Priority Rules | Allocate Constrained Product Supply | Allocate Exchange &amp; Third-Party Volumes</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Three allocation concepts coexist at different grains and are deliberately bounded here: plan-level placement (this node), order-level allocation and release (Order Management), and loading-time allocation enforcement (Terminal Loading). The “Decision” suffix is retained pending the same naming pass noted on CM-1-1-2-10.</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>Decide where available finished product is placed across markets, channels, and supply points to protect commitments and regional margin.</t>
+        </is>
+      </c>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>SRC-ASCM-CSCP-001 | SRC-SNF-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X12" s="5" t="n"/>
-      <c r="Y12" s="5" t="n"/>
-      <c r="Z12" s="5" t="n"/>
-      <c r="AA12" s="5" t="n"/>
-      <c r="AB12" s="5" t="n"/>
-      <c r="AC12" s="5" t="n"/>
+      <c r="Y12" s="5" t="inlineStr">
+        <is>
+          <t>demand forecast | available and planned production | inventory position | contractual and regulatory supply obligations | logistics and terminal capacity | netback and margin economics</t>
+        </is>
+      </c>
+      <c r="Z12" s="5" t="inlineStr">
+        <is>
+          <t>approved finished-product allocation plan by market, channel, and supply point</t>
+        </is>
+      </c>
+      <c r="AA12" s="5" t="inlineStr">
+        <is>
+          <t>informed-by: Demand Forecasting | constrained-by: Inventory | enables: Order Management | enables: Terminal Loading</t>
+        </is>
+      </c>
+      <c r="AB12" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC12" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1910,18 +2044,85 @@
           <t>strong APQC candidate but no validator agreed</t>
         </is>
       </c>
-      <c r="U13" s="5" t="n"/>
-      <c r="V13" s="5" t="n"/>
-      <c r="W13" s="5" t="n"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Create, maintain, and retire the reference and parameter data that the regional supply-planning model depends on — such as planning network, sourcing, capacity, lead-time, yield, and product-grouping data — so planning results remain accurate and reproducible.</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Covers stewardship of supply-planning-specific reference and parameter data over its lifecycle, including requesting and validating changes, applying effective dates, and confirming that planning results remain consistent after a change. Excludes enterprise master-data policy, standards, and governance, which sit with the Data Governance workstream; excludes customer, price, product, tax, and location master data, owned by Manage Master Data under Order Management; excludes production-scheduling master data, owned by Maintain Production Scheduling Master Data under Refinery Scheduling.</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Planning network and location data | sourcing and supply-path data | planning capacity and rate parameters | lead times and transit assumptions | planning yields and product groupings | change request, validation, and effective dating of planning parameters</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Enterprise master-data policy and governance standards (Data Governance) | customer, price, product, tax, and location master data (Manage Master Data, Order Management) | production-scheduling master data (Maintain Production Scheduling Master Data, Refinery Scheduling) | demand-forecast master data preparation (Prepare Master Data To Create Demand Forecast, Demand Forecasting) | planning application administration and platform support (Process Excellence &amp; IT)</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Supply Planning Reference Data Maintenance | Planning Parameter Maintenance</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Maintain Planning Network Data | Maintain Planning Capacity &amp; Rate Parameters | Maintain Planning Yield Data</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Defined narrowly per Hamid's decision (2026-09-18, Option 1): scope is the supply-planning-specific reference and parameter data consumed by the regional planning model, not master data generally. The taxonomy currently carries four parallel master-data nodes — this one, Maintain Production Scheduling Master Data (CM-1-1-7-2-1), Manage Master Data (CM-1-3-7-1), and Prepare Master Data To Create Demand Forecast (CM-1-1-1-1-1). Their consolidation, and whether a single governed master-data capability should own them, is parked for the EPM Data Governance workstream and is deliberately not resolved here. APQC candidate “Maintain master data” was triaged STRONG but accepted by no validator; used as comparative evidence only, not adopted.</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>Keep the reference and parameter data behind regional supply planning accurate, current, and reproducible.</t>
+        </is>
+      </c>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X13" s="5" t="n"/>
-      <c r="Y13" s="5" t="n"/>
-      <c r="Z13" s="5" t="n"/>
-      <c r="AA13" s="5" t="n"/>
-      <c r="AB13" s="5" t="n"/>
-      <c r="AC13" s="5" t="n"/>
+      <c r="Y13" s="5" t="inlineStr">
+        <is>
+          <t>planning parameter change requests | network, capacity, and sourcing changes | refinery and logistics capability updates | product and grade structure changes | enterprise data-governance standards</t>
+        </is>
+      </c>
+      <c r="Z13" s="5" t="inlineStr">
+        <is>
+          <t>validated and effective-dated supply-planning reference and parameter data</t>
+        </is>
+      </c>
+      <c r="AA13" s="5" t="inlineStr">
+        <is>
+          <t>enables: Regional Optimization | governed-by: Data Governance | informed-by: Refinery Planning</t>
+        </is>
+      </c>
+      <c r="AB13" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC13" s="5" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1989,18 +2190,85 @@
           <t>strong APQC candidate but no validator agreed</t>
         </is>
       </c>
-      <c r="U14" s="5" t="n"/>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="5" t="n"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Set and optimize the planned finished-product inventory levels and positions for the regional plan period, balancing supply availability, demand coverage, and working-capital cost within established inventory policy and storage constraints.</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Covers the planning decision on how much finished product should be held, in which grades, and at which supply points and terminals across the regional plan horizon, including target and minimum operating positions, seasonal and pre-build positions, and the inventory consequences of allocation and production choices. Excludes the setting of inventory policy itself, and excludes inventory measurement, reconciliation, replenishment, consignment, commingled, and re-brand inventory management, all owned by the Inventory cluster under Distribution Planning &amp; Scheduling. Excludes physical storage operation, owned by Midstream.</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Planned finished-product inventory targets by grade and location | minimum operating and safety positions within policy | seasonal and pre-build inventory positioning | inventory implications of allocation and production plan choices | working-capital and storage-cost trade-offs in the plan</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Finished-product inventory policy setting (Develop Finished Product Inventory Policy, Inventory) | inventory measurement and reconciliation (Inventory) | replenishment execution (Manage Inventory Replenishment, Inventory) | consignment, commingled, lot/batch, and re-brand inventory management (Inventory) | physical tank and terminal storage operation (Midstream)</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Finished Goods Inventory Planning | Finished Product Inventory Planning</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Set Regional Inventory Targets | Plan Seasonal Inventory Build | Plan Inventory for Constrained Supply</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Boundary resolved per Hamid's decision (2026-09-18, Option 1): this node owns the planned inventory level and position inside the regional plan, while the Inventory cluster under Distribution Planning &amp; Scheduling (CM-1-1-3-7) retains policy, measurement, reconciliation, and replenishment. This preserves both approved scope notes — Regional Optimization explicitly names “inventory positioning” — and the locked SCM rule, by separating the plan-period target decision from ongoing inventory management. No tree change required. “Finished goods” retained from the existing label although “finished product” is the more common downstream term; alt labels carry both.</t>
+        </is>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>Decide how much finished product should be held, in which grades, and where, across the regional plan horizon.</t>
+        </is>
+      </c>
+      <c r="W14" s="5" t="inlineStr">
+        <is>
+          <t>SRC-ASCM-CSCP-001 | SRC-SNF-REFPS-001</t>
+        </is>
+      </c>
       <c r="X14" s="5" t="n"/>
-      <c r="Y14" s="5" t="n"/>
-      <c r="Z14" s="5" t="n"/>
-      <c r="AA14" s="5" t="n"/>
-      <c r="AB14" s="5" t="n"/>
-      <c r="AC14" s="5" t="n"/>
+      <c r="Y14" s="5" t="inlineStr">
+        <is>
+          <t>demand forecast | planned production and supply availability | approved inventory policy | storage and terminal capacity | product specifications and seasonal grade changes | working-capital and storage-cost assumptions</t>
+        </is>
+      </c>
+      <c r="Z14" s="5" t="inlineStr">
+        <is>
+          <t>approved planned finished-product inventory targets and positions for the plan period</t>
+        </is>
+      </c>
+      <c r="AA14" s="5" t="inlineStr">
+        <is>
+          <t>constrained-by: Inventory | informed-by: Demand Forecasting | informed-by: Refinery Planning | enables: Product Allocation Decision</t>
+        </is>
+      </c>
+      <c r="AB14" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC14" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -4240,10 +4508,27 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U43" s="5" t="n"/>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>PARKED TREE CHANGE — no definition authored (2026-09-18). See business_architecture/ontology/step3c-parked-tree-changes.md, entry PTC-001, for the full proposal and the steps required to close it. This node carries no local meaning of its own: its three L5 children (Develop Strategic Business Plan, Plan Budgets, Manage Site Specific Business Risk) are not refinery production-planning activities, and Plan Budgets contradicts the locked rule that Finance owns financial governance. Authoring a definition here would silently endorse budgeting and strategic planning under Refinery Planning. Handled the same way as the parked IT Services reparenting question on CM-1, rather than churning the tree during a definition pass. The three L5 children are left untouched and remain pending.</t>
+        </is>
+      </c>
+      <c r="U43" s="5" t="inlineStr">
+        <is>
+          <t>mixed/needs-review</t>
+        </is>
+      </c>
       <c r="V43" s="5" t="n"/>
       <c r="W43" s="5" t="n"/>
-      <c r="X43" s="5" t="n"/>
+      <c r="X43" s="5" t="inlineStr">
+        <is>
+          <t>Question: Should "Commercial Development" remain a child of Refinery Planning, and if so, what is its scope?
+Context: Parent CM-1-1-4 Refinery Planning is approved as the commercially optimal refinery production plan (crude slate, throughput, yield, and specification targets). This node's three L5 children are Develop Strategic Business Plan (CM-1-1-4-6-1), Plan Budgets (CM-1-1-4-6-2), and Manage Site Specific Business Risk (CM-1-1-4-6-3). None is a refinery production-planning activity. Plan Budgets conflicts with the locked Finance boundary. The label itself came from a WEAK / REVIEW LINK APQC match ("Manage employee development") and carries no local meaning. Two of the three children have no existing owner in the tree: there is no Strategy node among the L1 domains, and the only risk nodes are Credit Risk and Market Risk under Supply And Trading, with EHS owning EHS risk only.
+Options: A) Retire the node from Refinery Planning, reparent Plan Budgets to Finance, and create two new nodes outside Planning &amp; Scheduling for the strategic-plan and site-risk children. B) Redefine narrowly as site commercial business development and reparent all three children elsewhere. C) Retire the node and reparent each child individually with no replacement parent.
+Evidence: Approved CM-1-1-4 definition and scope note; locked Finance and EHS boundary rules; Step 3b review_notes recording the weak APQC match; SRC-SNF-REFPS-001 on separation of strategic, planning, and scheduling horizons.
+Recommendation: Option A, parked as a tree-change proposal for the consolidated repo-JSON pass rather than a definition authored now. Accepted by Hamid 2026-09-18; tracked as PTC-001 in step3c-parked-tree-changes.md.</t>
+        </is>
+      </c>
       <c r="Y43" s="5" t="n"/>
       <c r="Z43" s="5" t="n"/>
       <c r="AA43" s="5" t="n"/>
@@ -4556,18 +4841,85 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U47" s="5" t="n"/>
-      <c r="V47" s="5" t="n"/>
-      <c r="W47" s="5" t="n"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Run the recurring economic-optimization cycle that produces the refinery production plan — assembling the case basis, building and running optimization cases, analyzing scenarios, and selecting the economically preferred production case for approval.</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Covers the optimization cycle inside Refinery Planning: gathering the demand, crude availability, price, constraint, inventory, and current-plan basis for a case; building and running the optimization model; comparing alternatives through scenario analysis; and recommending the economically preferred case. Accountability for the approved production plan and its commercial targets remains with Refinery Planning. Excludes detailed unit-operation scheduling, tank and transfer line-ups, blend execution, and process control, owned by Refining; excludes optimization-model and application administration, owned by Process Excellence &amp; IT.</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Assemble case basis from demand, crude availability, price, constraints, inventory, and current plan | build and run optimization cases | scenario and sensitivity analysis | compare production alternatives on margin | recommend the economically preferred production case</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Approval and ownership of the production plan and its commercial targets (Refinery Planning) | detailed unit scheduling, tank line-ups, and blend execution (Refining, Refinery Scheduling) | process control and operational departures from plan (Refining) | optimization application administration and model platform support (Process Excellence &amp; IT) | real-time and closed-loop unit optimization (Refining)</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Refinery Economic Optimization | Refinery Plan Optimization | Refinery LP Optimization</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Build Optimization Case | Validate Case Basis | Recommend Preferred Production Case</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Parent-versus-child distinctness resolved per Hamid's decision (2026-09-18, Option 1): Refinery Planning (CM-1-1-4) owns the approved plan and its commercial targets; this node owns the recurring optimization run cycle that produces the candidate plan. Without that split the two primary purposes were near-identical. The eight existing L5 children — six “Capture …” nodes, Evaluate Crude &amp; Feedstock, and Perform Scenario Analysis — are coherent under this reading as case-basis assembly and case analysis. “Capture Monthly Operating Plan” (CM-1-1-4-7-7) appears to name a document rather than a process and is flagged for review in the L5 batch, not resolved here. Avoided naming a specific optimization application; “LP” appears only as an alternate label because it is established industry shorthand.</t>
+        </is>
+      </c>
+      <c r="U47" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V47" s="5" t="inlineStr">
+        <is>
+          <t>Produce and recommend the economically preferred refinery production case for the planning period.</t>
+        </is>
+      </c>
+      <c r="W47" s="5" t="inlineStr">
+        <is>
+          <t>SRC-CMU-REFPLAN-001 | SRC-SNF-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X47" s="5" t="n"/>
-      <c r="Y47" s="5" t="n"/>
-      <c r="Z47" s="5" t="n"/>
-      <c r="AA47" s="5" t="n"/>
-      <c r="AB47" s="5" t="n"/>
-      <c r="AC47" s="5" t="n"/>
+      <c r="Y47" s="5" t="inlineStr">
+        <is>
+          <t>product demand requirements | crude and feedstock availability and assays | crude, feedstock, and product prices | refinery capacity and operating constraints | inventory position | current approved operating plan</t>
+        </is>
+      </c>
+      <c r="Z47" s="5" t="inlineStr">
+        <is>
+          <t>recommended economically preferred refinery production case with supporting scenario analysis</t>
+        </is>
+      </c>
+      <c r="AA47" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Planning | informed-by: Demand Forecasting | informed-by: Crude Allocation Decision | constrained-by: Inventory | precedes: Refinery Scheduling</t>
+        </is>
+      </c>
+      <c r="AB47" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC47" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -41166,7 +41518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41544,8 +41896,196 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>U.S. Energy Information Administration</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Glossary and petroleum table definitions</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/tools/glossary/</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Government statistical authority</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Standard US downstream terminology; evidence only, not text to copy</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Refinery, crude slate, capacity, and product-category terminology</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Association for Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>CSCP Exam Content Manual</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Current edition, accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ascm.org/globalassets/ascm_website_assets/docs/ecm/ecm-cscp.pdf</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Professional standards body</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Supply-chain planning terminology; evidence only</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Allocation, master-data, inventory-planning, and S&amp;OP terminology</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SRC-CMU-REFPLAN-001</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University (Su, Grossmann et al.)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Modeling for Integrated Refinery Planning with Crude-oil Scheduling</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>https://egon.cheme.cmu.edu/Papers/Su_IntegratedRefineryPlanning.pdf</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Peer-reviewed academic</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Planning-versus-scheduling decision separation; evidence only</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Crude allocation, slate selection, and refinery optimization cycle</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>SRC-SNF-REFPS-001</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Institute for Research in Economics and Business Administration (SNF)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Refinery planning and scheduling</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Report R29/08, accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>https://snf.no/media/2uvkatl3/r29_08.pdf</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Academic research institute</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Planning hierarchy and horizon separation; evidence only</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Strategic, planning, and scheduling horizon boundaries in refining</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:I13"/>
+  <autoFilter ref="A7:I17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Step 3c: review batch 01 — Regional Optimization & Refinery Planning (#32)
Co-authored-by: aadehamid <7918263+aadehamid@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
+++ b/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review &amp; authoring'!$A$1:$AD$504</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Controlled vocabularies'!$A$3:$C$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Reference register'!$A$7:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Reference register'!$A$7:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'External mappings'!$A$8:$K$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1752,18 +1752,85 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U11" s="5" t="n"/>
-      <c r="V11" s="5" t="n"/>
-      <c r="W11" s="5" t="n"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Assign available crude and feedstock cargoes, grades, and volumes to specific refineries and receipt windows so each site's approved production plan can be met at the best delivered economics across the region.</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Covers the recurring allocation of secured or available crude and feedstock supply across competing refinery destinations, including grade-to-site matching, volume splits, timing of receipt windows, and reallocation when supply or plan assumptions change. Excludes crude purchase, negotiation, and trade execution, owned by Supply And Trading; excludes vessel, pipeline, and terminal movement execution, owned by Midstream; excludes the refinery's internal decision on which tanks and units process an allocated grade, owned by Refining.</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Grade-to-refinery assignment | volume split across sites | receipt-window timing | reallocation on supply disruption or plan change | allocation of term and spot volumes against planned refinery slates</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Crude purchasing and trade execution (Supply And Trading) | physical movement, berth and pipeline scheduling (Midstream) | unit-level crude processing decisions (Refining) | refinery slate economics selection (Refinery Planning)</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Crude Allocation | Feedstock Allocation | Crude &amp; Feedstock Allocation</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Allocate Term Crude Volumes | Allocate Spot Crude Volumes | Reallocate Crude on Supply Disruption</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Label retains the existing “Decision” suffix, but the concept is authored as the recurring allocation process, not the decision record or its output. A later naming pass should consider “Allocate Crude &amp; Feedstock” for verb consistency with sibling labels; not changed in this batch. The boundary against Supply And Trading follows the locked SCM/Commercial rule: this concept places already-secured supply and does not choose counterparty, price, or contract.</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>Decide which refinery receives which crude and feedstock volumes, and when, so the regional plan is met at best delivered economics.</t>
+        </is>
+      </c>
+      <c r="W11" s="5" t="inlineStr">
+        <is>
+          <t>SRC-CMU-REFPLAN-001 | SRC-SNF-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X11" s="5" t="n"/>
-      <c r="Y11" s="5" t="n"/>
-      <c r="Z11" s="5" t="n"/>
-      <c r="AA11" s="5" t="n"/>
-      <c r="AB11" s="5" t="n"/>
-      <c r="AC11" s="5" t="n"/>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
+          <t>approved refinery production plan | secured and available crude supply position | crude and feedstock quality assays | delivered-cost and freight economics | refinery receipt and storage constraints</t>
+        </is>
+      </c>
+      <c r="Z11" s="5" t="inlineStr">
+        <is>
+          <t>approved crude and feedstock allocation to refineries and receipt windows</t>
+        </is>
+      </c>
+      <c r="AA11" s="5" t="inlineStr">
+        <is>
+          <t>informed-by: Refinery Planning | constrained-by: Inventory | precedes: Refinery Scheduling</t>
+        </is>
+      </c>
+      <c r="AB11" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC11" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1831,18 +1898,85 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U12" s="5" t="n"/>
-      <c r="V12" s="5" t="n"/>
-      <c r="W12" s="5" t="n"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Assign available finished-product supply to markets, channels, terminals, and customer commitments for a planning period, so limited or constrained volumes are placed where they best serve contractual obligations and regional margin.</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Covers plan-level placement of finished product across markets, channels, and supply points, including the commercial priority rules applied when available supply cannot meet all demand, and reallocation when supply, demand, or logistics change. Excludes order-level allocation and release against an individual customer order, owned by Order Management; excludes rack and terminal loading allocation enforcement, owned by Terminal Loading; excludes physical movement and delivery execution, owned by Midstream and Distribution.</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Market and channel volume placement | supply-point-to-demand-point assignment | commercial priority rules under constrained supply | exchange and third-party placement within the plan | reallocation on plan change</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Order-level allocation and release (Allocate &amp; Release Order, Order Management) | rack and terminal allocation enforcement (Manage Allocation, Terminal Loading) | sales-target setting (Determine &amp; Allocate Sales Targets, Marketing) | pricing and offer construction (Commercial &amp; Marketing pricing processes) | physical delivery (Midstream, Distribution)</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Product Allocation | Finished Product Allocation | Supply Allocation</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Define Product Allocation Priority Rules | Allocate Constrained Product Supply | Allocate Exchange &amp; Third-Party Volumes</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Three allocation concepts coexist at different grains and are deliberately bounded here: plan-level placement (this node), order-level allocation and release (Order Management), and loading-time allocation enforcement (Terminal Loading). The “Decision” suffix is retained pending the same naming pass noted on CM-1-1-2-10.</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>Decide where available finished product is placed across markets, channels, and supply points to protect commitments and regional margin.</t>
+        </is>
+      </c>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>SRC-ASCM-CSCP-001 | SRC-SNF-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X12" s="5" t="n"/>
-      <c r="Y12" s="5" t="n"/>
-      <c r="Z12" s="5" t="n"/>
-      <c r="AA12" s="5" t="n"/>
-      <c r="AB12" s="5" t="n"/>
-      <c r="AC12" s="5" t="n"/>
+      <c r="Y12" s="5" t="inlineStr">
+        <is>
+          <t>demand forecast | available and planned production | inventory position | contractual and regulatory supply obligations | logistics and terminal capacity | netback and margin economics</t>
+        </is>
+      </c>
+      <c r="Z12" s="5" t="inlineStr">
+        <is>
+          <t>approved finished-product allocation plan by market, channel, and supply point</t>
+        </is>
+      </c>
+      <c r="AA12" s="5" t="inlineStr">
+        <is>
+          <t>informed-by: Demand Forecasting | constrained-by: Inventory | enables: Order Management | enables: Terminal Loading</t>
+        </is>
+      </c>
+      <c r="AB12" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC12" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1910,18 +2044,85 @@
           <t>strong APQC candidate but no validator agreed</t>
         </is>
       </c>
-      <c r="U13" s="5" t="n"/>
-      <c r="V13" s="5" t="n"/>
-      <c r="W13" s="5" t="n"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Create, maintain, and retire the reference and parameter data that the regional supply-planning model depends on — such as planning network, sourcing, capacity, lead-time, yield, and product-grouping data — so planning results remain accurate and reproducible.</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Covers stewardship of supply-planning-specific reference and parameter data over its lifecycle, including requesting and validating changes, applying effective dates, and confirming that planning results remain consistent after a change. Excludes enterprise master-data policy, standards, and governance, which sit with the Data Governance workstream; excludes customer, price, product, tax, and location master data, owned by Manage Master Data under Order Management; excludes production-scheduling master data, owned by Maintain Production Scheduling Master Data under Refinery Scheduling.</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Planning network and location data | sourcing and supply-path data | planning capacity and rate parameters | lead times and transit assumptions | planning yields and product groupings | change request, validation, and effective dating of planning parameters</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Enterprise master-data policy and governance standards (Data Governance) | customer, price, product, tax, and location master data (Manage Master Data, Order Management) | production-scheduling master data (Maintain Production Scheduling Master Data, Refinery Scheduling) | demand-forecast master data preparation (Prepare Master Data To Create Demand Forecast, Demand Forecasting) | planning application administration and platform support (Process Excellence &amp; IT)</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Supply Planning Reference Data Maintenance | Planning Parameter Maintenance</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Maintain Planning Network Data | Maintain Planning Capacity &amp; Rate Parameters | Maintain Planning Yield Data</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Defined narrowly per Hamid's decision (2026-09-18, Option 1): scope is the supply-planning-specific reference and parameter data consumed by the regional planning model, not master data generally. The taxonomy currently carries four parallel master-data nodes — this one, Maintain Production Scheduling Master Data (CM-1-1-7-2-1), Manage Master Data (CM-1-3-7-1), and Prepare Master Data To Create Demand Forecast (CM-1-1-1-1-1). Their consolidation, and whether a single governed master-data capability should own them, is parked for the EPM Data Governance workstream and is deliberately not resolved here. APQC candidate “Maintain master data” was triaged STRONG but accepted by no validator; used as comparative evidence only, not adopted.</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>Keep the reference and parameter data behind regional supply planning accurate, current, and reproducible.</t>
+        </is>
+      </c>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X13" s="5" t="n"/>
-      <c r="Y13" s="5" t="n"/>
-      <c r="Z13" s="5" t="n"/>
-      <c r="AA13" s="5" t="n"/>
-      <c r="AB13" s="5" t="n"/>
-      <c r="AC13" s="5" t="n"/>
+      <c r="Y13" s="5" t="inlineStr">
+        <is>
+          <t>planning parameter change requests | network, capacity, and sourcing changes | refinery and logistics capability updates | product and grade structure changes | enterprise data-governance standards</t>
+        </is>
+      </c>
+      <c r="Z13" s="5" t="inlineStr">
+        <is>
+          <t>validated and effective-dated supply-planning reference and parameter data</t>
+        </is>
+      </c>
+      <c r="AA13" s="5" t="inlineStr">
+        <is>
+          <t>enables: Regional Optimization | governed-by: Data Governance | informed-by: Refinery Planning</t>
+        </is>
+      </c>
+      <c r="AB13" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC13" s="5" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1989,18 +2190,85 @@
           <t>strong APQC candidate but no validator agreed</t>
         </is>
       </c>
-      <c r="U14" s="5" t="n"/>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="5" t="n"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Set and optimize the planned finished-product inventory levels and positions for the regional plan period, balancing supply availability, demand coverage, and working-capital cost within established inventory policy and storage constraints.</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Covers the planning decision on how much finished product should be held, in which grades, and at which supply points and terminals across the regional plan horizon, including target and minimum operating positions, seasonal and pre-build positions, and the inventory consequences of allocation and production choices. Excludes the setting of inventory policy itself, and excludes inventory measurement, reconciliation, replenishment, consignment, commingled, and re-brand inventory management, all owned by the Inventory cluster under Distribution Planning &amp; Scheduling. Excludes physical storage operation, owned by Midstream.</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Planned finished-product inventory targets by grade and location | minimum operating and safety positions within policy | seasonal and pre-build inventory positioning | inventory implications of allocation and production plan choices | working-capital and storage-cost trade-offs in the plan</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Finished-product inventory policy setting (Develop Finished Product Inventory Policy, Inventory) | inventory measurement and reconciliation (Inventory) | replenishment execution (Manage Inventory Replenishment, Inventory) | consignment, commingled, lot/batch, and re-brand inventory management (Inventory) | physical tank and terminal storage operation (Midstream)</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Finished Goods Inventory Planning | Finished Product Inventory Planning</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Set Regional Inventory Targets | Plan Seasonal Inventory Build | Plan Inventory for Constrained Supply</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Boundary resolved per Hamid's decision (2026-09-18, Option 1): this node owns the planned inventory level and position inside the regional plan, while the Inventory cluster under Distribution Planning &amp; Scheduling (CM-1-1-3-7) retains policy, measurement, reconciliation, and replenishment. This preserves both approved scope notes — Regional Optimization explicitly names “inventory positioning” — and the locked SCM rule, by separating the plan-period target decision from ongoing inventory management. No tree change required. “Finished goods” retained from the existing label although “finished product” is the more common downstream term; alt labels carry both.</t>
+        </is>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>Decide how much finished product should be held, in which grades, and where, across the regional plan horizon.</t>
+        </is>
+      </c>
+      <c r="W14" s="5" t="inlineStr">
+        <is>
+          <t>SRC-ASCM-CSCP-001 | SRC-SNF-REFPS-001</t>
+        </is>
+      </c>
       <c r="X14" s="5" t="n"/>
-      <c r="Y14" s="5" t="n"/>
-      <c r="Z14" s="5" t="n"/>
-      <c r="AA14" s="5" t="n"/>
-      <c r="AB14" s="5" t="n"/>
-      <c r="AC14" s="5" t="n"/>
+      <c r="Y14" s="5" t="inlineStr">
+        <is>
+          <t>demand forecast | planned production and supply availability | approved inventory policy | storage and terminal capacity | product specifications and seasonal grade changes | working-capital and storage-cost assumptions</t>
+        </is>
+      </c>
+      <c r="Z14" s="5" t="inlineStr">
+        <is>
+          <t>approved planned finished-product inventory targets and positions for the plan period</t>
+        </is>
+      </c>
+      <c r="AA14" s="5" t="inlineStr">
+        <is>
+          <t>constrained-by: Inventory | informed-by: Demand Forecasting | informed-by: Refinery Planning | enables: Product Allocation Decision</t>
+        </is>
+      </c>
+      <c r="AB14" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC14" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -4240,10 +4508,27 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U43" s="5" t="n"/>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>PARKED TREE CHANGE — no definition authored (2026-09-18). See business_architecture/ontology/step3c-parked-tree-changes.md, entry PTC-001, for the full proposal and the steps required to close it. This node carries no local meaning of its own: its three L5 children (Develop Strategic Business Plan, Plan Budgets, Manage Site Specific Business Risk) are not refinery production-planning activities, and Plan Budgets contradicts the locked rule that Finance owns financial governance. Authoring a definition here would silently endorse budgeting and strategic planning under Refinery Planning. Handled the same way as the parked IT Services reparenting question on CM-1, rather than churning the tree during a definition pass. The three L5 children are left untouched and remain pending.</t>
+        </is>
+      </c>
+      <c r="U43" s="5" t="inlineStr">
+        <is>
+          <t>mixed/needs-review</t>
+        </is>
+      </c>
       <c r="V43" s="5" t="n"/>
       <c r="W43" s="5" t="n"/>
-      <c r="X43" s="5" t="n"/>
+      <c r="X43" s="5" t="inlineStr">
+        <is>
+          <t>Question: Should "Commercial Development" remain a child of Refinery Planning, and if so, what is its scope?
+Context: Parent CM-1-1-4 Refinery Planning is approved as the commercially optimal refinery production plan (crude slate, throughput, yield, and specification targets). This node's three L5 children are Develop Strategic Business Plan (CM-1-1-4-6-1), Plan Budgets (CM-1-1-4-6-2), and Manage Site Specific Business Risk (CM-1-1-4-6-3). None is a refinery production-planning activity. Plan Budgets conflicts with the locked Finance boundary. The label itself came from a WEAK / REVIEW LINK APQC match ("Manage employee development") and carries no local meaning. Two of the three children have no existing owner in the tree: there is no Strategy node among the L1 domains, and the only risk nodes are Credit Risk and Market Risk under Supply And Trading, with EHS owning EHS risk only.
+Options: A) Retire the node from Refinery Planning, reparent Plan Budgets to Finance, and create two new nodes outside Planning &amp; Scheduling for the strategic-plan and site-risk children. B) Redefine narrowly as site commercial business development and reparent all three children elsewhere. C) Retire the node and reparent each child individually with no replacement parent.
+Evidence: Approved CM-1-1-4 definition and scope note; locked Finance and EHS boundary rules; Step 3b review_notes recording the weak APQC match; SRC-SNF-REFPS-001 on separation of strategic, planning, and scheduling horizons.
+Recommendation: Option A, parked as a tree-change proposal for the consolidated repo-JSON pass rather than a definition authored now. Accepted by Hamid 2026-09-18; tracked as PTC-001 in step3c-parked-tree-changes.md.</t>
+        </is>
+      </c>
       <c r="Y43" s="5" t="n"/>
       <c r="Z43" s="5" t="n"/>
       <c r="AA43" s="5" t="n"/>
@@ -4556,18 +4841,85 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U47" s="5" t="n"/>
-      <c r="V47" s="5" t="n"/>
-      <c r="W47" s="5" t="n"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Run the recurring economic-optimization cycle that produces the refinery production plan — assembling the case basis, building and running optimization cases, analyzing scenarios, and selecting the economically preferred production case for approval.</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Covers the optimization cycle inside Refinery Planning: gathering the demand, crude availability, price, constraint, inventory, and current-plan basis for a case; building and running the optimization model; comparing alternatives through scenario analysis; and recommending the economically preferred case. Accountability for the approved production plan and its commercial targets remains with Refinery Planning. Excludes detailed unit-operation scheduling, tank and transfer line-ups, blend execution, and process control, owned by Refining; excludes optimization-model and application administration, owned by Process Excellence &amp; IT.</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Assemble case basis from demand, crude availability, price, constraints, inventory, and current plan | build and run optimization cases | scenario and sensitivity analysis | compare production alternatives on margin | recommend the economically preferred production case</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Approval and ownership of the production plan and its commercial targets (Refinery Planning) | detailed unit scheduling, tank line-ups, and blend execution (Refining, Refinery Scheduling) | process control and operational departures from plan (Refining) | optimization application administration and model platform support (Process Excellence &amp; IT) | real-time and closed-loop unit optimization (Refining)</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Refinery Economic Optimization | Refinery Plan Optimization | Refinery LP Optimization</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Build Optimization Case | Validate Case Basis | Recommend Preferred Production Case</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Parent-versus-child distinctness resolved per Hamid's decision (2026-09-18, Option 1): Refinery Planning (CM-1-1-4) owns the approved plan and its commercial targets; this node owns the recurring optimization run cycle that produces the candidate plan. Without that split the two primary purposes were near-identical. The eight existing L5 children — six “Capture …” nodes, Evaluate Crude &amp; Feedstock, and Perform Scenario Analysis — are coherent under this reading as case-basis assembly and case analysis. “Capture Monthly Operating Plan” (CM-1-1-4-7-7) appears to name a document rather than a process and is flagged for review in the L5 batch, not resolved here. Avoided naming a specific optimization application; “LP” appears only as an alternate label because it is established industry shorthand.</t>
+        </is>
+      </c>
+      <c r="U47" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V47" s="5" t="inlineStr">
+        <is>
+          <t>Produce and recommend the economically preferred refinery production case for the planning period.</t>
+        </is>
+      </c>
+      <c r="W47" s="5" t="inlineStr">
+        <is>
+          <t>SRC-CMU-REFPLAN-001 | SRC-SNF-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X47" s="5" t="n"/>
-      <c r="Y47" s="5" t="n"/>
-      <c r="Z47" s="5" t="n"/>
-      <c r="AA47" s="5" t="n"/>
-      <c r="AB47" s="5" t="n"/>
-      <c r="AC47" s="5" t="n"/>
+      <c r="Y47" s="5" t="inlineStr">
+        <is>
+          <t>product demand requirements | crude and feedstock availability and assays | crude, feedstock, and product prices | refinery capacity and operating constraints | inventory position | current approved operating plan</t>
+        </is>
+      </c>
+      <c r="Z47" s="5" t="inlineStr">
+        <is>
+          <t>recommended economically preferred refinery production case with supporting scenario analysis</t>
+        </is>
+      </c>
+      <c r="AA47" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Planning | informed-by: Demand Forecasting | informed-by: Crude Allocation Decision | constrained-by: Inventory | precedes: Refinery Scheduling</t>
+        </is>
+      </c>
+      <c r="AB47" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC47" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -41166,7 +41518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41544,8 +41896,196 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>U.S. Energy Information Administration</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Glossary and petroleum table definitions</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/tools/glossary/</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Government statistical authority</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Standard US downstream terminology; evidence only, not text to copy</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Refinery, crude slate, capacity, and product-category terminology</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Association for Supply Chain Management</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>CSCP Exam Content Manual</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Current edition, accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ascm.org/globalassets/ascm_website_assets/docs/ecm/ecm-cscp.pdf</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Professional standards body</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Supply-chain planning terminology; evidence only</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Allocation, master-data, inventory-planning, and S&amp;OP terminology</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SRC-CMU-REFPLAN-001</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University (Su, Grossmann et al.)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Modeling for Integrated Refinery Planning with Crude-oil Scheduling</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>https://egon.cheme.cmu.edu/Papers/Su_IntegratedRefineryPlanning.pdf</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Peer-reviewed academic</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Planning-versus-scheduling decision separation; evidence only</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Crude allocation, slate selection, and refinery optimization cycle</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>SRC-SNF-REFPS-001</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Institute for Research in Economics and Business Administration (SNF)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Refinery planning and scheduling</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Report R29/08, accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>https://snf.no/media/2uvkatl3/r29_08.pdf</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Academic research institute</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Planning hierarchy and horizon separation; evidence only</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Strategic, planning, and scheduling horizon boundaries in refining</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:I13"/>
+  <autoFilter ref="A7:I17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Step 3c: sync reviewer guide and validator to semantic-intake workbook
Same follow-up as #30 after #29: #31/#32 changed the workbook contract
and left the locked guide plus mechanical gate on the old 2-sheet,
pending|approved-only rules.

- Lock step3c-reviewer-instructions.md at v2026-09-19 (6 sheets, Phase 1/2,
  blocked/retired, PTC register, open_questions protocol).
- Validator enforces the new contract. The 15 #29 approvals are listed in
  PRE_INTAKE_APPROVED — empty Phase 1 is NOTE, not silent and not blocking.
  CM-1-3-3-5-6 missing scope_note stays blocking.
- Playbook §7 and the 3c step log record why. Column guide rows that still
  required a sibling owner were rewritten to the #30 locked rule.

No JSON/TTL/RDF emission. No Phase 1 backfill on the 15.

Co-authored-by: Hamid Adesokan <aadehamid@gmail.com>
</commit_message>
<xml_diff>
--- a/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
+++ b/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review &amp; authoring'!$A$1:$AD$504</definedName>
@@ -40991,6 +40991,11 @@
           <t>skos:definition (required on every concept; @en)</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Phase 1 — required</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -41000,12 +41005,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Coverage list + boundary sentences: what it includes, what it explicitly excludes, and which sibling owns the excluded part.</t>
+          <t>Coverage plus at least one meaningful boundary. Name exclusions and owners only when ambiguity is material and the owner is already in the taxonomy. Do not manufacture boilerplate exclusions.</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
           <t>skos:scopeNote (@en)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Phase 1 — required</t>
         </is>
       </c>
     </row>
@@ -41025,6 +41035,11 @@
           <t>folded into skos:scopeNote</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Phase 1 — supporting</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -41034,12 +41049,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Activities/cases that do NOT belong here + who owns them instead — feeds the scope note's exclusion list.</t>
+          <t>Activities or cases that do not belong here. Name the owning sibling or domain only when it is already established. Otherwise ask in open_questions and leave pending.</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
           <t>folded into skos:scopeNote</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Phase 1 — supporting</t>
         </is>
       </c>
     </row>
@@ -41059,6 +41079,11 @@
           <t>skos:altLabel (@en)</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Phase 1 — supporting</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -41068,12 +41093,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Future narrower concepts spotted while defining, separated by |. Become new nodes in a later modeling pass.</t>
+          <t>Future narrower concepts spotted while defining, separated by |. Become new nodes in a later modeling pass. Tree moves of existing nodes go in step3c-parked-tree-changes.md, not here.</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
           <t>future skos:narrower concepts; consolidated repo-JSON proposal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Phase 1 — supporting</t>
         </is>
       </c>
     </row>
@@ -41085,12 +41115,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Wording decisions (e.g. 'production horizons' not 'run schedules') so they don't get reopened.</t>
+          <t>Wording and modeling decisions (e.g. 'production horizons' not 'run schedules') so they don't get reopened. Structured questions for Hamid go in open_questions.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
           <t>editorial note in the decision log / JSON record</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Phase 1 — supporting</t>
         </is>
       </c>
     </row>
@@ -41102,12 +41137,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>pending → approved. Only approved rows merge into the taxonomy.</t>
+          <t>pending → approved when the row passes all checks. blocked / retired only after Hamid parks or a PTC retires the node. Only approved rows merge.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
           <t>workflow control; merged via step3-skos-taxonomy.py --authored</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Workflow — pending | approved | blocked | retired</t>
         </is>
       </c>
     </row>
@@ -41132,6 +41172,11 @@
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Semantic-intake fields added in the Step 3c intake evolution</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Added in #31. Required on new approvals. The 15 #29 approved rows are grandfathered until a later backfill; the validator flags them as NOTE, not BLOCKING. RDF is not emitted from these fields yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Step 3c: review batch 02 — Refinery Optimization L5, plus gate-blocker and heuristic fixes
Bundle A: batch 02, the 8 L5 children of CM-1-1-4-7. Seven approved, CM-1-1-4-7-7 held pending with a structured question. PTC-002 raised.
Bundle B: scope_note added to CM-1-3-3-5-6, clearing the last BLOCKING gate finding from #30.
Bundle C: circular-opening and out-of-scope-owner heuristics in step3c-workbook-validate.py retargeted; 10 false QUESTIONs and 5 false NOTEs removed, real faults still caught.
</commit_message>
<xml_diff>
--- a/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
+++ b/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review &amp; authoring'!$A$1:$AD$504</definedName>
@@ -4987,18 +4987,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U48" s="5" t="n"/>
-      <c r="V48" s="5" t="n"/>
-      <c r="W48" s="5" t="n"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Assemble the demand requirements that the refinery production case must satisfy — by product, volume, quality grade, location, and delivery period — drawing on the approved demand forecast, firm contractual commitments, and internal transfer requirements for the planning period.</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Covers converting demand signals into the demand basis of an optimization case: selecting the applicable forecast version, adding firm contractual and internal transfer obligations, reconciling units and product grades to planning definitions, and confirming the basis with the demand owner. Excludes producing or owning the forecast itself, which belongs to Demand Forecasting (CM-1-1-1-1) and Refined Product Demand Management (CM-1-2-6-2). Excludes capturing or committing customer orders, owned by Order Management (CM-1-3-7).</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Select the applicable approved demand forecast version | add firm contractual and term commitments | add internal and inter-refinery transfer requirements | reconcile product grades, units, and periods to planning definitions | confirm the agreed demand basis for the case</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Producing or owning the demand forecast, owned by Demand Forecasting (CM-1-1-1-1) | forecasting refined product demand, owned by Forecast Refined Product Demand (CM-1-2-6-2-3) | capturing and committing customer orders, owned by Order Management (CM-1-3-7) | negotiating the underlying customer commitment, owned by Commercial &amp; Marketing sales | placing supply against demand, owned by Product Allocation Decision (CM-1-1-2-11)</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Capture Demand Basis | Establish Product Demand Requirements | Demand Basis Capture</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. “Requirements” is read as the obligations the plan must meet, not as product specification requirements. Verb kept as the taxonomy label “Capture”; “Receive Demand Forecast” (CM-1-2-1-1-2) is the existing precedent for a consume-not-produce node.</t>
+        </is>
+      </c>
+      <c r="U48" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V48" s="5" t="inlineStr">
+        <is>
+          <t>Establish the agreed demand basis the refinery production case must satisfy.</t>
+        </is>
+      </c>
+      <c r="W48" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X48" s="5" t="n"/>
-      <c r="Y48" s="5" t="n"/>
-      <c r="Z48" s="5" t="n"/>
-      <c r="AA48" s="5" t="n"/>
-      <c r="AB48" s="5" t="n"/>
-      <c r="AC48" s="5" t="n"/>
+      <c r="Y48" s="5" t="inlineStr">
+        <is>
+          <t>approved demand forecast | firm contracts and term commitments | internal and inter-refinery transfer requirements | product grade and specification definitions</t>
+        </is>
+      </c>
+      <c r="Z48" s="5" t="inlineStr">
+        <is>
+          <t>agreed product demand basis for the refinery optimization case</t>
+        </is>
+      </c>
+      <c r="AA48" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | informed-by: Demand Forecasting | informed-by: Refined Product Demand Management | precedes: Perform Scenario Analysis</t>
+        </is>
+      </c>
+      <c r="AB48" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC48" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD48" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5066,18 +5128,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U49" s="5" t="n"/>
-      <c r="V49" s="5" t="n"/>
-      <c r="W49" s="5" t="n"/>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Assess candidate crude oils and feedstocks for processing suitability and economic value in the planning period, using assay and quality data, expected yields against the refinery configuration, and delivered-cost economics, to produce the evaluated set available to the optimization case.</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Covers technical and economic screening of candidate crudes and feedstocks for planning: confirming assay and quality data is current and complete, estimating yields and processing fit against unit configuration and specification limits, valuing each candidate on a delivered-cost and netback basis, and flagging handling or compatibility issues. Excludes laboratory assay testing and certification, and excludes purchase, negotiation, and trade execution, owned by Supply And Trading (CM-1-2). Approval of the final crude slate remains with Refinery Planning (CM-1-1-4).</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Confirm assay and quality data currency and completeness | estimate yields and processing fit against refinery configuration | screen against specification and handling limits | value candidates on delivered cost and netback | rank and publish the evaluated crude and feedstock set</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Purchasing, negotiating, and executing crude and feedstock trades, owned by Supply And Trading (CM-1-2) | laboratory assay testing and certification, owned by Refining laboratory services | approving the final crude slate, owned by Refinery Planning (CM-1-1-4) | placing secured crude across refineries, owned by Crude Allocation Decision (CM-1-1-2-10) | crude and feedstock master data stewardship, owned by Manage feedstock Data Quality (CM-1-2-5-1-1)</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Evaluate Crude &amp; Feedstock Slate Candidates | Crude Assay Evaluation | Crude Screening</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. Boundary against “Plan Optimal Feedstock Slate And Run Rate” (CM-1-2-5-2-3) under Supply And Trading is unresolved: on its label that node duplicates the approved Refinery Planning accountability for slate and throughput targets. Raised as PTC-002 in step3c-parked-tree-changes.md and deliberately not reconciled here, since resolving it is a tree change. This node is bounded as evaluation only, so it does not depend on that outcome.</t>
+        </is>
+      </c>
+      <c r="U49" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V49" s="5" t="inlineStr">
+        <is>
+          <t>Produce the technically and economically evaluated crude and feedstock set for the planning period.</t>
+        </is>
+      </c>
+      <c r="W49" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-CMU-REFPLAN-001</t>
+        </is>
+      </c>
       <c r="X49" s="5" t="n"/>
-      <c r="Y49" s="5" t="n"/>
-      <c r="Z49" s="5" t="n"/>
-      <c r="AA49" s="5" t="n"/>
-      <c r="AB49" s="5" t="n"/>
-      <c r="AC49" s="5" t="n"/>
+      <c r="Y49" s="5" t="inlineStr">
+        <is>
+          <t>crude and feedstock assays and quality data | refinery configuration and unit capability | product specification limits | delivered cost, freight, and differential data | candidate supply offers</t>
+        </is>
+      </c>
+      <c r="Z49" s="5" t="inlineStr">
+        <is>
+          <t>evaluated and ranked crude and feedstock set with yield and value estimates</t>
+        </is>
+      </c>
+      <c r="AA49" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | uses-input: Capture Crude Availability | uses-input: Capture Product/Crude/Feedstock Price | constrained-by: Capture Refinery Level Constraints</t>
+        </is>
+      </c>
+      <c r="AB49" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC49" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD49" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5145,18 +5269,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U50" s="5" t="n"/>
-      <c r="V50" s="5" t="n"/>
-      <c r="W50" s="5" t="n"/>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Establish which crude and feedstock volumes can realistically be secured and delivered inside the planning period — by grade, source, and arrival window — covering already-contracted supply, term liftings, and credible spot opportunities.</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Covers the supply-side volume basis of an optimization case: confirming contracted and term volumes, identifying credible additional spot availability, and stating arrival windows and any logistics or quality qualifications. Establishes what is available, not what is bought or where it is sent. Excludes securing supply and executing trades, owned by Supply And Trading (CM-1-2); excludes arrival and delivery scheduling, owned by Plan Feedstock Arrival (CM-1-2-5-3-3); excludes placing secured supply across refineries, owned by Crude Allocation Decision (CM-1-1-2-10).</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Confirm contracted and term supply volumes and lifting windows | identify credible incremental spot availability | state arrival windows and delivery qualifications | flag logistics, quality, or compatibility limits on availability | publish the available supply basis for the case</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Securing, negotiating, and executing supply, owned by Supply And Trading (CM-1-2) | scheduling arrivals and deliveries, owned by Plan Feedstock Arrival (CM-1-2-5-3-3) and Schedule Feedstock Delivery (CM-1-2-5-3-2) | placing secured crude across refineries, owned by Crude Allocation Decision (CM-1-1-2-10) | judging processing suitability or value, owned by Evaluate Crude &amp; Feedstock (CM-1-1-4-7-2) | managing feedstock inventory, owned by Manage Feedstock Inventory (CM-1-2-5-4-2)</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Capture Crude &amp; Feedstock Availability | Establish Supply Availability | Crude Availability Basis</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. Availability is the volume-and-timing basis; suitability and value sit in Evaluate Crude &amp; Feedstock (CM-1-1-4-7-2), and the placement decision sits in the approved Crude Allocation Decision (CM-1-1-2-10). The taxonomy label says “Crude”; feedstock is included because the sibling optimization basis and the parent scope both treat them together.</t>
+        </is>
+      </c>
+      <c r="U50" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V50" s="5" t="inlineStr">
+        <is>
+          <t>Establish the crude and feedstock volumes and arrival windows available to the planning period.</t>
+        </is>
+      </c>
+      <c r="W50" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X50" s="5" t="n"/>
-      <c r="Y50" s="5" t="n"/>
-      <c r="Z50" s="5" t="n"/>
-      <c r="AA50" s="5" t="n"/>
-      <c r="AB50" s="5" t="n"/>
-      <c r="AC50" s="5" t="n"/>
+      <c r="Y50" s="5" t="inlineStr">
+        <is>
+          <t>term and spot supply contracts | lifting and nomination schedules | supplier availability advice | marine and pipeline logistics availability | port and tankage receipt limits</t>
+        </is>
+      </c>
+      <c r="Z50" s="5" t="inlineStr">
+        <is>
+          <t>available crude and feedstock supply basis by grade, source, and arrival window</t>
+        </is>
+      </c>
+      <c r="AA50" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | enables: Evaluate Crude &amp; Feedstock | informed-by: Supply And Trading | constrained-by: Capture Refinery Level Constraints</t>
+        </is>
+      </c>
+      <c r="AB50" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC50" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD50" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5224,18 +5410,80 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U51" s="5" t="n"/>
-      <c r="V51" s="5" t="n"/>
-      <c r="W51" s="5" t="n"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Establish the price and economic assumption set used to value crude, feedstock, and finished-product streams in the optimization case — market reference prices, quality and location differentials, freight, and internal transfer values — for the planning period.</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Covers assembling and confirming the planning price basis: selecting reference quotations and forward curves, applying grade and location differentials and freight, setting internal transfer and intermediate stream values, and recording the assumption set so a case can be reproduced and later backcast. These are planning assumptions, not transactable prices. Excludes setting customer sales prices, owned by Sales Pricing Management (CM-1-3-6-3); excludes pricing strategy, owned by Pricing Strategy Management (CM-1-3-3-2); excludes price master data, owned by Maintain Price &amp; Discount Master Data (CM-1-3-7-1-2).</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Select reference price quotations and forward curves | apply quality, grade, and location differentials | apply freight and delivery cost assumptions | set internal transfer and intermediate stream values | record and version the price assumption set for the case</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Setting and implementing customer sales prices, owned by Sales Pricing Management (CM-1-3-6-3) | pricing strategy and approach, owned by Pricing Strategy Management (CM-1-3-3-2) | price and discount master data stewardship, owned by Maintain Price &amp; Discount Master Data (CM-1-3-7-1-2) | price risk management and hedging, owned by Supply And Trading (CM-1-2-2) | transaction and invoice pricing, owned by Finance</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Capture Planning Price Basis | Establish Price Assumptions | Price Assumption Capture</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. The distinction that matters is assumption versus transaction: this node sets the prices a case is evaluated against, while the Marketing and Sales pricing nodes set prices a customer actually pays. The recorded assumption set is also the contemporaneous basis the locked backcasting rule requires, since Regional and Distribution Backcasting compare actuals to the approved plan and its original assumptions, never a later reforecast.</t>
+        </is>
+      </c>
+      <c r="U51" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V51" s="5" t="inlineStr">
+        <is>
+          <t>Establish the reproducible price and economic assumption set used to value the optimization case.</t>
+        </is>
+      </c>
+      <c r="W51" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X51" s="5" t="n"/>
-      <c r="Y51" s="5" t="n"/>
-      <c r="Z51" s="5" t="n"/>
-      <c r="AA51" s="5" t="n"/>
-      <c r="AB51" s="5" t="n"/>
-      <c r="AC51" s="5" t="n"/>
+      <c r="Y51" s="5" t="inlineStr">
+        <is>
+          <t>published market quotations and forward curves | quality and location differentials | freight and logistics cost rates | internal transfer pricing policy | operating cost assumptions</t>
+        </is>
+      </c>
+      <c r="Z51" s="5" t="inlineStr">
+        <is>
+          <t>versioned price and economic assumption set for the planning period</t>
+        </is>
+      </c>
+      <c r="AA51" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | enables: Evaluate Crude &amp; Feedstock | informed-by: Supply And Trading | produces: contemporaneous assumption basis for Regional Backcasting</t>
+        </is>
+      </c>
+      <c r="AB51" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC51" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5303,18 +5551,80 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U52" s="5" t="n"/>
-      <c r="V52" s="5" t="n"/>
-      <c r="W52" s="5" t="n"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Compile the limits a refinery production case must respect — unit capacities and rates, blending and product-specification limits, tankage and movement limits, and planned maintenance or turnaround outages — as the feasible operating envelope for the planning period.</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Covers gathering, validating, and stating constraints in planning terms: confirming available unit capacity and rate limits including outage-adjusted availability, recording specification and blending limits, recording tankage and movement limits, and reconciling conflicting or stale limits with the constraint owner. Compiles limits set elsewhere; it does not set them. Excludes deciding maintenance and turnaround scope and timing, and excludes operating-limit ownership and process control, both owned by Refining. Excludes regulatory and permit limit ownership, owned by EHS &amp; Gov Reporting.</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Confirm unit capacity, rate, and outage-adjusted availability | record product specification and blending limits | record tankage, movement, and logistics limits | record contractual and regulatory volume limits as planning constraints | reconcile stale or conflicting limits with the constraint owner | publish the case operating envelope</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Setting and owning unit operating limits and process control, owned by Refining | deciding maintenance and turnaround scope and timing, owned by Refining maintenance planning | owning regulatory, permit, and emissions limits, owned by EHS &amp; Gov Reporting | setting product specifications as an offer decision, owned by Offer Design &amp; Development (CM-1-3-3) | detailed unit scheduling within the envelope, owned by Refining</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Capture Refinery Constraints | Establish Operating Envelope | Constraint Basis Capture</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. “Refinery level” is read as site-wide rather than unit-detail granularity, consistent with the locked boundary that Refinery Planning sets commercial production-plan targets while Refining owns detailed scheduling and execution. Compiling a constraint does not transfer ownership of it.</t>
+        </is>
+      </c>
+      <c r="U52" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V52" s="5" t="inlineStr">
+        <is>
+          <t>Establish the validated feasible operating envelope the production case must respect.</t>
+        </is>
+      </c>
+      <c r="W52" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-CMU-REFPLAN-001</t>
+        </is>
+      </c>
       <c r="X52" s="5" t="n"/>
-      <c r="Y52" s="5" t="n"/>
-      <c r="Z52" s="5" t="n"/>
-      <c r="AA52" s="5" t="n"/>
-      <c r="AB52" s="5" t="n"/>
-      <c r="AC52" s="5" t="n"/>
+      <c r="Y52" s="5" t="inlineStr">
+        <is>
+          <t>unit capacity and rate limits | planned maintenance and turnaround schedule | product specification and blending limits | tankage, jetty, and pipeline capacity | regulatory, permit, and contractual limits</t>
+        </is>
+      </c>
+      <c r="Z52" s="5" t="inlineStr">
+        <is>
+          <t>validated refinery operating envelope and constraint set for the case</t>
+        </is>
+      </c>
+      <c r="AA52" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | constrained-by: Refining | informed-by: EHS &amp; Gov Reporting | constrains: Perform Scenario Analysis</t>
+        </is>
+      </c>
+      <c r="AB52" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC52" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD52" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5377,18 +5687,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U53" s="5" t="n"/>
-      <c r="V53" s="5" t="n"/>
-      <c r="W53" s="5" t="n"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Establish the inventory position the optimization case starts from and the closing position it must deliver — crude, intermediate, and finished-product volumes by location and grade — including any volume that is unavailable to the plan.</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Covers stating inventory as a planning boundary condition: taking the opening position from the system of record, adjusting for in-transit and committed volume, separating working stock from unavailable volume such as tank bottoms, minimum operating stock, and consignment or commingled volume, and carrying in the required closing target. Excludes measuring and reconciling inventory, owned by Measure Inventory (CM-1-1-3-7-4) and Perform Inventory Reconciliation (CM-1-1-3-7-5). Excludes inventory policy, owned by the Inventory cluster (CM-1-1-3-7). Excludes setting the plan-period finished-goods target, owned by Plan Finished Goods Inventory (CM-1-1-2-13).</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Take the opening inventory position from the system of record | adjust for in-transit and already-committed volume | separate working stock from unavailable volume | carry in the required closing inventory target | state inventory assumptions and qualifications for the case</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Measuring, counting, and reconciling inventory, owned by Measure Inventory (CM-1-1-3-7-4) and Perform Inventory Reconciliation (CM-1-1-3-7-5) | setting inventory policy, owned by the Inventory cluster (CM-1-1-3-7) | setting the plan-period finished-goods target and position, owned by Plan Finished Goods Inventory (CM-1-1-2-13) | day-to-day stock and replenishment management, owned by Manage Inventory Replenishment (CM-1-1-3-7-9) | inventory valuation and accounting, owned by Finance</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Capture Inventory Position | Establish Opening Inventory | Inventory Basis Capture</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. Three inventory nodes are now distinct and must stay that way: this node states the position as a case boundary condition, Plan Finished Goods Inventory (CM-1-1-2-13, approved) sets the plan-period target, and the Inventory cluster (CM-1-1-3-7) owns policy, measurement, reconciliation, and replenishment. The bare taxonomy label “Capture Inventory” is the weakest of the eight and “Capture Inventory Position” is recorded as the preferred alternate label.</t>
+        </is>
+      </c>
+      <c r="U53" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V53" s="5" t="inlineStr">
+        <is>
+          <t>Establish the opening and required closing inventory position bounding the optimization case.</t>
+        </is>
+      </c>
+      <c r="W53" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X53" s="5" t="n"/>
-      <c r="Y53" s="5" t="n"/>
-      <c r="Z53" s="5" t="n"/>
-      <c r="AA53" s="5" t="n"/>
-      <c r="AB53" s="5" t="n"/>
-      <c r="AC53" s="5" t="n"/>
+      <c r="Y53" s="5" t="inlineStr">
+        <is>
+          <t>inventory system of record position | in-transit and committed volumes | minimum operating and unavailable stock levels | plan-period finished-goods inventory target | tankage and segregation constraints</t>
+        </is>
+      </c>
+      <c r="Z53" s="5" t="inlineStr">
+        <is>
+          <t>opening and required closing inventory basis for the optimization case</t>
+        </is>
+      </c>
+      <c r="AA53" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | uses-input: Plan Finished Goods Inventory | informed-by: Measure Inventory | constrained-by: Inventory</t>
+        </is>
+      </c>
+      <c r="AB53" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC53" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD53" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5456,10 +5828,22 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U54" s="5" t="n"/>
+      <c r="U54" s="5" t="inlineStr">
+        <is>
+          <t>mixed/needs-review</t>
+        </is>
+      </c>
       <c r="V54" s="5" t="n"/>
       <c r="W54" s="5" t="n"/>
-      <c r="X54" s="5" t="n"/>
+      <c r="X54" s="5" t="inlineStr">
+        <is>
+          <t>Question: Is “Capture Monthly Operating Plan” a process, or does it name the monthly operating plan document itself?
+Context: The seven sibling L5 nodes under Refinery Optimization (CM-1-1-4-7) partition the case basis and its analysis. The monthly operating plan is the output of the optimization cycle, not an input to it, so on a plain reading this node inverts the direction of the sibling set. Its Step 3b APQC candidate was “Plan facility”, scored NONE / NO CANDIDATE, so there is no external signal either way.
+Options: (1) Define it as issuing and registering the approved monthly operating plan as the plan of record handed to Refining for scheduling — a real process, and it closes the optimization cycle; no tree change needed, rename to “Issue Monthly Operating Plan” as preferred label. (2) Define it as loading the current approved operating plan as the starting baseline for the next case — also a real process and a genuine input, but it overlaps the parent scope phrase “current approved operating plan” already covered in the case basis. (3) Classify as not-process, a document rather than an activity, and retire the node; the plan artifact is then represented as the primary_output of CM-1-1-4-7 and CM-1-1-4. (4) Split: keep an issue step here and represent the plan artifact as an output, not a node.
+Evidence: SRC-BJCE-REFPS-001 describes monthly rolling plans as the product of tactical refinery planning, which assigns production targets to process units, and separates planning from scheduling; SRC-SNF-REFPS-001 and SRC-CMU-REFPLAN-001 place the plan as the handover from planning to scheduling. All three support the plan being an output of this cycle, none supports it being captured as an input.
+Recommendation: Option 1. It is the only reading that makes the node a process, leaves the tree unchanged, and gives the optimization cycle an explicit handover step to Refining, which the locked Refining boundary implies but no current node carries. Option 3 is the honest alternative if you would rather not re-point a label. Not defining the row until you decide, because Options 1 and 3 differ on whether the node survives.</t>
+        </is>
+      </c>
       <c r="Y54" s="5" t="n"/>
       <c r="Z54" s="5" t="n"/>
       <c r="AA54" s="5" t="n"/>
@@ -5535,18 +5919,80 @@
           <t>strong APQC candidate but no validator agreed</t>
         </is>
       </c>
-      <c r="U55" s="5" t="n"/>
-      <c r="V55" s="5" t="n"/>
-      <c r="W55" s="5" t="n"/>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Compare alternative production cases by varying crude slate, run rates, product mix, price, or constraint assumptions, and quantify the margin and feasibility consequences of each, so the preferred case and its sensitivities are understood before the plan is approved.</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Covers case-based analysis inside the optimization cycle: defining the scenarios worth testing, running them against the case basis, reading marginal values and binding constraints, quantifying margin and feasibility differences, and documenting the comparison that supports the recommended case. Excludes selecting and approving the production plan, owned by Refinery Planning (CM-1-1-4). Excludes trading and market risk scenarios, owned by Manage And Run Risk Scenarios (CM-1-2-2-3-11). Excludes comparing actual performance to the approved plan, owned by Regional Backcasting (CM-1-1-5) and Distribution Backcasting (CM-1-1-6).</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Define the scenarios and sensitivities worth testing | run alternative cases against the case basis | read marginal values and identify binding constraints | quantify margin, yield, and feasibility differences | document the case comparison supporting the recommendation</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Selecting and approving the production plan, owned by Refinery Planning (CM-1-1-4) | trading and market risk scenarios, owned by Manage And Run Risk Scenarios (CM-1-2-2-3-11) | comparing actuals to the approved plan, owned by Regional Backcasting (CM-1-1-5) and Distribution Backcasting (CM-1-1-6) | investment and strategic configuration studies | optimization model and application administration, owned by Process Excellence &amp; IT</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Perform Case &amp; Sensitivity Analysis | Run Optimization Scenarios | Case Comparison</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node is the analysis step rather than a case-basis input. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. Scenario analysis here is forward-looking case comparison within a planning period. It is distinct from backcasting, which is retrospective, and from trading risk scenarios, which test market exposure rather than production alternatives. The APQC candidate “Perform competitive analysis” scored STRONG but is about comparing bidder proposals and was rejected as a false lexical match.</t>
+        </is>
+      </c>
+      <c r="U55" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V55" s="5" t="inlineStr">
+        <is>
+          <t>Quantify and compare production alternatives and their sensitivities to support case selection.</t>
+        </is>
+      </c>
+      <c r="W55" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-CMU-REFPLAN-001 | SRC-SNF-REFPS-001</t>
+        </is>
+      </c>
       <c r="X55" s="5" t="n"/>
-      <c r="Y55" s="5" t="n"/>
-      <c r="Z55" s="5" t="n"/>
-      <c r="AA55" s="5" t="n"/>
-      <c r="AB55" s="5" t="n"/>
-      <c r="AC55" s="5" t="n"/>
+      <c r="Y55" s="5" t="inlineStr">
+        <is>
+          <t>assembled case basis of demand, availability, price, constraints, and inventory | base optimization case and solution | candidate scenario definitions | marginal values and binding constraint output</t>
+        </is>
+      </c>
+      <c r="Z55" s="5" t="inlineStr">
+        <is>
+          <t>documented case comparison with margin, feasibility, and sensitivity results</t>
+        </is>
+      </c>
+      <c r="AA55" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | uses-input: Capture Product Demand Requirements | uses-input: Capture Refinery Level Constraints | precedes: Refinery Planning</t>
+        </is>
+      </c>
+      <c r="AB55" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC55" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD55" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -25316,6 +25762,16 @@
       <c r="N307" t="inlineStr">
         <is>
           <t>Developing a program to promote the objectives, values, products and services of the company to its employees by treating them as potential customers, in order to extend company client base, increase employee engagement or to foster brand advocacy.</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>Covers setting the strategy for communicating brand, offer, and marketing messages to the organization's own employees as an internal audience: audience and channel choice, message and tone direction, and the intended engagement or advocacy outcome. Strategy only. Excludes executing internal communications, owned by Implement Internal Communications (CM-1-3-5-3-9), and excludes campaign-level planning, owned by Marketing Communications Planning (CM-1-3-5-3). Excludes external, media, public, investor, and government communications, which the locked Legal &amp; Corp Comm boundary places outside this branch. Excludes employee relations, terms of employment, and HR policy communication.</t>
+        </is>
+      </c>
+      <c r="T307" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18), bundled fix. Row was approved in the #29 pre-intake pass with an empty scope_note and has been the single BLOCKING finding of step3c-workbook-validate.py since #30. Only the missing scope_note was added; the approved definition, status, and all other fields are unchanged. Boundaries asserted here are drawn from existing taxonomy siblings and the locked Legal &amp; Corp Comm decision, not from new research. Phase 1 fields remain empty, consistent with this row staying on the PRE_INTAKE_APPROVED allowlist for the later backfill pass.</t>
         </is>
       </c>
       <c r="U307" s="5" t="n"/>
@@ -41563,7 +42019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -42124,6 +42580,100 @@
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>U.S. Energy Information Administration (DiVita)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Liquid Fuels Market Module refinery LP modeling white paper</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/outlooks/documentation/workshops/pdf/VDiVita%20LFMM%20White%20Paper.pdf</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Government statistical authority</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Refinery LP input categories and model structure; evidence only, not text to copy</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Refinery optimization case basis: assays, availability, prices, specifications, capacities</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SRC-BJCE-REFPS-001</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Brazilian Journal of Chemical Engineering (Moro)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Refinery production planning and scheduling: the refining coordination case</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.scielo.br/j/bjce/a/GMRKZJGQ5HPqWRPfwKxnWTq/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Peer-reviewed academic</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Planning-versus-scheduling separation and monthly rolling plan evidence; evidence only</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Case-basis inputs, monthly operating plan as planning output, sensitivity analysis</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
Step 3c: review batch 02 — Refinery Optimization L5, plus gate-blocker and heuristic fixes (#34)
Bundle A: batch 02, the 8 L5 children of CM-1-1-4-7. Seven approved, CM-1-1-4-7-7 held pending with a structured question. PTC-002 raised.
Bundle B: scope_note added to CM-1-3-3-5-6, clearing the last BLOCKING gate finding from #30.
Bundle C: circular-opening and out-of-scope-owner heuristics in step3c-workbook-validate.py retargeted; 10 false QUESTIONs and 5 false NOTEs removed, real faults still caught.

Co-authored-by: aadehamid <7918263+aadehamid@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
+++ b/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review &amp; authoring'!$A$1:$AD$504</definedName>
@@ -4987,18 +4987,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U48" s="5" t="n"/>
-      <c r="V48" s="5" t="n"/>
-      <c r="W48" s="5" t="n"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Assemble the demand requirements that the refinery production case must satisfy — by product, volume, quality grade, location, and delivery period — drawing on the approved demand forecast, firm contractual commitments, and internal transfer requirements for the planning period.</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Covers converting demand signals into the demand basis of an optimization case: selecting the applicable forecast version, adding firm contractual and internal transfer obligations, reconciling units and product grades to planning definitions, and confirming the basis with the demand owner. Excludes producing or owning the forecast itself, which belongs to Demand Forecasting (CM-1-1-1-1) and Refined Product Demand Management (CM-1-2-6-2). Excludes capturing or committing customer orders, owned by Order Management (CM-1-3-7).</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Select the applicable approved demand forecast version | add firm contractual and term commitments | add internal and inter-refinery transfer requirements | reconcile product grades, units, and periods to planning definitions | confirm the agreed demand basis for the case</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Producing or owning the demand forecast, owned by Demand Forecasting (CM-1-1-1-1) | forecasting refined product demand, owned by Forecast Refined Product Demand (CM-1-2-6-2-3) | capturing and committing customer orders, owned by Order Management (CM-1-3-7) | negotiating the underlying customer commitment, owned by Commercial &amp; Marketing sales | placing supply against demand, owned by Product Allocation Decision (CM-1-1-2-11)</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Capture Demand Basis | Establish Product Demand Requirements | Demand Basis Capture</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. “Requirements” is read as the obligations the plan must meet, not as product specification requirements. Verb kept as the taxonomy label “Capture”; “Receive Demand Forecast” (CM-1-2-1-1-2) is the existing precedent for a consume-not-produce node.</t>
+        </is>
+      </c>
+      <c r="U48" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V48" s="5" t="inlineStr">
+        <is>
+          <t>Establish the agreed demand basis the refinery production case must satisfy.</t>
+        </is>
+      </c>
+      <c r="W48" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X48" s="5" t="n"/>
-      <c r="Y48" s="5" t="n"/>
-      <c r="Z48" s="5" t="n"/>
-      <c r="AA48" s="5" t="n"/>
-      <c r="AB48" s="5" t="n"/>
-      <c r="AC48" s="5" t="n"/>
+      <c r="Y48" s="5" t="inlineStr">
+        <is>
+          <t>approved demand forecast | firm contracts and term commitments | internal and inter-refinery transfer requirements | product grade and specification definitions</t>
+        </is>
+      </c>
+      <c r="Z48" s="5" t="inlineStr">
+        <is>
+          <t>agreed product demand basis for the refinery optimization case</t>
+        </is>
+      </c>
+      <c r="AA48" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | informed-by: Demand Forecasting | informed-by: Refined Product Demand Management | precedes: Perform Scenario Analysis</t>
+        </is>
+      </c>
+      <c r="AB48" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC48" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD48" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5066,18 +5128,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U49" s="5" t="n"/>
-      <c r="V49" s="5" t="n"/>
-      <c r="W49" s="5" t="n"/>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Assess candidate crude oils and feedstocks for processing suitability and economic value in the planning period, using assay and quality data, expected yields against the refinery configuration, and delivered-cost economics, to produce the evaluated set available to the optimization case.</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Covers technical and economic screening of candidate crudes and feedstocks for planning: confirming assay and quality data is current and complete, estimating yields and processing fit against unit configuration and specification limits, valuing each candidate on a delivered-cost and netback basis, and flagging handling or compatibility issues. Excludes laboratory assay testing and certification, and excludes purchase, negotiation, and trade execution, owned by Supply And Trading (CM-1-2). Approval of the final crude slate remains with Refinery Planning (CM-1-1-4).</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Confirm assay and quality data currency and completeness | estimate yields and processing fit against refinery configuration | screen against specification and handling limits | value candidates on delivered cost and netback | rank and publish the evaluated crude and feedstock set</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Purchasing, negotiating, and executing crude and feedstock trades, owned by Supply And Trading (CM-1-2) | laboratory assay testing and certification, owned by Refining laboratory services | approving the final crude slate, owned by Refinery Planning (CM-1-1-4) | placing secured crude across refineries, owned by Crude Allocation Decision (CM-1-1-2-10) | crude and feedstock master data stewardship, owned by Manage feedstock Data Quality (CM-1-2-5-1-1)</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Evaluate Crude &amp; Feedstock Slate Candidates | Crude Assay Evaluation | Crude Screening</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. Boundary against “Plan Optimal Feedstock Slate And Run Rate” (CM-1-2-5-2-3) under Supply And Trading is unresolved: on its label that node duplicates the approved Refinery Planning accountability for slate and throughput targets. Raised as PTC-002 in step3c-parked-tree-changes.md and deliberately not reconciled here, since resolving it is a tree change. This node is bounded as evaluation only, so it does not depend on that outcome.</t>
+        </is>
+      </c>
+      <c r="U49" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V49" s="5" t="inlineStr">
+        <is>
+          <t>Produce the technically and economically evaluated crude and feedstock set for the planning period.</t>
+        </is>
+      </c>
+      <c r="W49" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-CMU-REFPLAN-001</t>
+        </is>
+      </c>
       <c r="X49" s="5" t="n"/>
-      <c r="Y49" s="5" t="n"/>
-      <c r="Z49" s="5" t="n"/>
-      <c r="AA49" s="5" t="n"/>
-      <c r="AB49" s="5" t="n"/>
-      <c r="AC49" s="5" t="n"/>
+      <c r="Y49" s="5" t="inlineStr">
+        <is>
+          <t>crude and feedstock assays and quality data | refinery configuration and unit capability | product specification limits | delivered cost, freight, and differential data | candidate supply offers</t>
+        </is>
+      </c>
+      <c r="Z49" s="5" t="inlineStr">
+        <is>
+          <t>evaluated and ranked crude and feedstock set with yield and value estimates</t>
+        </is>
+      </c>
+      <c r="AA49" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | uses-input: Capture Crude Availability | uses-input: Capture Product/Crude/Feedstock Price | constrained-by: Capture Refinery Level Constraints</t>
+        </is>
+      </c>
+      <c r="AB49" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC49" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD49" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5145,18 +5269,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U50" s="5" t="n"/>
-      <c r="V50" s="5" t="n"/>
-      <c r="W50" s="5" t="n"/>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Establish which crude and feedstock volumes can realistically be secured and delivered inside the planning period — by grade, source, and arrival window — covering already-contracted supply, term liftings, and credible spot opportunities.</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Covers the supply-side volume basis of an optimization case: confirming contracted and term volumes, identifying credible additional spot availability, and stating arrival windows and any logistics or quality qualifications. Establishes what is available, not what is bought or where it is sent. Excludes securing supply and executing trades, owned by Supply And Trading (CM-1-2); excludes arrival and delivery scheduling, owned by Plan Feedstock Arrival (CM-1-2-5-3-3); excludes placing secured supply across refineries, owned by Crude Allocation Decision (CM-1-1-2-10).</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Confirm contracted and term supply volumes and lifting windows | identify credible incremental spot availability | state arrival windows and delivery qualifications | flag logistics, quality, or compatibility limits on availability | publish the available supply basis for the case</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Securing, negotiating, and executing supply, owned by Supply And Trading (CM-1-2) | scheduling arrivals and deliveries, owned by Plan Feedstock Arrival (CM-1-2-5-3-3) and Schedule Feedstock Delivery (CM-1-2-5-3-2) | placing secured crude across refineries, owned by Crude Allocation Decision (CM-1-1-2-10) | judging processing suitability or value, owned by Evaluate Crude &amp; Feedstock (CM-1-1-4-7-2) | managing feedstock inventory, owned by Manage Feedstock Inventory (CM-1-2-5-4-2)</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Capture Crude &amp; Feedstock Availability | Establish Supply Availability | Crude Availability Basis</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. Availability is the volume-and-timing basis; suitability and value sit in Evaluate Crude &amp; Feedstock (CM-1-1-4-7-2), and the placement decision sits in the approved Crude Allocation Decision (CM-1-1-2-10). The taxonomy label says “Crude”; feedstock is included because the sibling optimization basis and the parent scope both treat them together.</t>
+        </is>
+      </c>
+      <c r="U50" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V50" s="5" t="inlineStr">
+        <is>
+          <t>Establish the crude and feedstock volumes and arrival windows available to the planning period.</t>
+        </is>
+      </c>
+      <c r="W50" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X50" s="5" t="n"/>
-      <c r="Y50" s="5" t="n"/>
-      <c r="Z50" s="5" t="n"/>
-      <c r="AA50" s="5" t="n"/>
-      <c r="AB50" s="5" t="n"/>
-      <c r="AC50" s="5" t="n"/>
+      <c r="Y50" s="5" t="inlineStr">
+        <is>
+          <t>term and spot supply contracts | lifting and nomination schedules | supplier availability advice | marine and pipeline logistics availability | port and tankage receipt limits</t>
+        </is>
+      </c>
+      <c r="Z50" s="5" t="inlineStr">
+        <is>
+          <t>available crude and feedstock supply basis by grade, source, and arrival window</t>
+        </is>
+      </c>
+      <c r="AA50" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | enables: Evaluate Crude &amp; Feedstock | informed-by: Supply And Trading | constrained-by: Capture Refinery Level Constraints</t>
+        </is>
+      </c>
+      <c r="AB50" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC50" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD50" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5224,18 +5410,80 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U51" s="5" t="n"/>
-      <c r="V51" s="5" t="n"/>
-      <c r="W51" s="5" t="n"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Establish the price and economic assumption set used to value crude, feedstock, and finished-product streams in the optimization case — market reference prices, quality and location differentials, freight, and internal transfer values — for the planning period.</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Covers assembling and confirming the planning price basis: selecting reference quotations and forward curves, applying grade and location differentials and freight, setting internal transfer and intermediate stream values, and recording the assumption set so a case can be reproduced and later backcast. These are planning assumptions, not transactable prices. Excludes setting customer sales prices, owned by Sales Pricing Management (CM-1-3-6-3); excludes pricing strategy, owned by Pricing Strategy Management (CM-1-3-3-2); excludes price master data, owned by Maintain Price &amp; Discount Master Data (CM-1-3-7-1-2).</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Select reference price quotations and forward curves | apply quality, grade, and location differentials | apply freight and delivery cost assumptions | set internal transfer and intermediate stream values | record and version the price assumption set for the case</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Setting and implementing customer sales prices, owned by Sales Pricing Management (CM-1-3-6-3) | pricing strategy and approach, owned by Pricing Strategy Management (CM-1-3-3-2) | price and discount master data stewardship, owned by Maintain Price &amp; Discount Master Data (CM-1-3-7-1-2) | price risk management and hedging, owned by Supply And Trading (CM-1-2-2) | transaction and invoice pricing, owned by Finance</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Capture Planning Price Basis | Establish Price Assumptions | Price Assumption Capture</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. The distinction that matters is assumption versus transaction: this node sets the prices a case is evaluated against, while the Marketing and Sales pricing nodes set prices a customer actually pays. The recorded assumption set is also the contemporaneous basis the locked backcasting rule requires, since Regional and Distribution Backcasting compare actuals to the approved plan and its original assumptions, never a later reforecast.</t>
+        </is>
+      </c>
+      <c r="U51" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V51" s="5" t="inlineStr">
+        <is>
+          <t>Establish the reproducible price and economic assumption set used to value the optimization case.</t>
+        </is>
+      </c>
+      <c r="W51" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-EIA-GLOSS-001</t>
+        </is>
+      </c>
       <c r="X51" s="5" t="n"/>
-      <c r="Y51" s="5" t="n"/>
-      <c r="Z51" s="5" t="n"/>
-      <c r="AA51" s="5" t="n"/>
-      <c r="AB51" s="5" t="n"/>
-      <c r="AC51" s="5" t="n"/>
+      <c r="Y51" s="5" t="inlineStr">
+        <is>
+          <t>published market quotations and forward curves | quality and location differentials | freight and logistics cost rates | internal transfer pricing policy | operating cost assumptions</t>
+        </is>
+      </c>
+      <c r="Z51" s="5" t="inlineStr">
+        <is>
+          <t>versioned price and economic assumption set for the planning period</t>
+        </is>
+      </c>
+      <c r="AA51" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | enables: Evaluate Crude &amp; Feedstock | informed-by: Supply And Trading | produces: contemporaneous assumption basis for Regional Backcasting</t>
+        </is>
+      </c>
+      <c r="AB51" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC51" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5303,18 +5551,80 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U52" s="5" t="n"/>
-      <c r="V52" s="5" t="n"/>
-      <c r="W52" s="5" t="n"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Compile the limits a refinery production case must respect — unit capacities and rates, blending and product-specification limits, tankage and movement limits, and planned maintenance or turnaround outages — as the feasible operating envelope for the planning period.</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Covers gathering, validating, and stating constraints in planning terms: confirming available unit capacity and rate limits including outage-adjusted availability, recording specification and blending limits, recording tankage and movement limits, and reconciling conflicting or stale limits with the constraint owner. Compiles limits set elsewhere; it does not set them. Excludes deciding maintenance and turnaround scope and timing, and excludes operating-limit ownership and process control, both owned by Refining. Excludes regulatory and permit limit ownership, owned by EHS &amp; Gov Reporting.</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Confirm unit capacity, rate, and outage-adjusted availability | record product specification and blending limits | record tankage, movement, and logistics limits | record contractual and regulatory volume limits as planning constraints | reconcile stale or conflicting limits with the constraint owner | publish the case operating envelope</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Setting and owning unit operating limits and process control, owned by Refining | deciding maintenance and turnaround scope and timing, owned by Refining maintenance planning | owning regulatory, permit, and emissions limits, owned by EHS &amp; Gov Reporting | setting product specifications as an offer decision, owned by Offer Design &amp; Development (CM-1-3-3) | detailed unit scheduling within the envelope, owned by Refining</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Capture Refinery Constraints | Establish Operating Envelope | Constraint Basis Capture</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. “Refinery level” is read as site-wide rather than unit-detail granularity, consistent with the locked boundary that Refinery Planning sets commercial production-plan targets while Refining owns detailed scheduling and execution. Compiling a constraint does not transfer ownership of it.</t>
+        </is>
+      </c>
+      <c r="U52" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V52" s="5" t="inlineStr">
+        <is>
+          <t>Establish the validated feasible operating envelope the production case must respect.</t>
+        </is>
+      </c>
+      <c r="W52" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-CMU-REFPLAN-001</t>
+        </is>
+      </c>
       <c r="X52" s="5" t="n"/>
-      <c r="Y52" s="5" t="n"/>
-      <c r="Z52" s="5" t="n"/>
-      <c r="AA52" s="5" t="n"/>
-      <c r="AB52" s="5" t="n"/>
-      <c r="AC52" s="5" t="n"/>
+      <c r="Y52" s="5" t="inlineStr">
+        <is>
+          <t>unit capacity and rate limits | planned maintenance and turnaround schedule | product specification and blending limits | tankage, jetty, and pipeline capacity | regulatory, permit, and contractual limits</t>
+        </is>
+      </c>
+      <c r="Z52" s="5" t="inlineStr">
+        <is>
+          <t>validated refinery operating envelope and constraint set for the case</t>
+        </is>
+      </c>
+      <c r="AA52" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | constrained-by: Refining | informed-by: EHS &amp; Gov Reporting | constrains: Perform Scenario Analysis</t>
+        </is>
+      </c>
+      <c r="AB52" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC52" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD52" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5377,18 +5687,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U53" s="5" t="n"/>
-      <c r="V53" s="5" t="n"/>
-      <c r="W53" s="5" t="n"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Establish the inventory position the optimization case starts from and the closing position it must deliver — crude, intermediate, and finished-product volumes by location and grade — including any volume that is unavailable to the plan.</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Covers stating inventory as a planning boundary condition: taking the opening position from the system of record, adjusting for in-transit and committed volume, separating working stock from unavailable volume such as tank bottoms, minimum operating stock, and consignment or commingled volume, and carrying in the required closing target. Excludes measuring and reconciling inventory, owned by Measure Inventory (CM-1-1-3-7-4) and Perform Inventory Reconciliation (CM-1-1-3-7-5). Excludes inventory policy, owned by the Inventory cluster (CM-1-1-3-7). Excludes setting the plan-period finished-goods target, owned by Plan Finished Goods Inventory (CM-1-1-2-13).</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Take the opening inventory position from the system of record | adjust for in-transit and already-committed volume | separate working stock from unavailable volume | carry in the required closing inventory target | state inventory assumptions and qualifications for the case</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Measuring, counting, and reconciling inventory, owned by Measure Inventory (CM-1-1-3-7-4) and Perform Inventory Reconciliation (CM-1-1-3-7-5) | setting inventory policy, owned by the Inventory cluster (CM-1-1-3-7) | setting the plan-period finished-goods target and position, owned by Plan Finished Goods Inventory (CM-1-1-2-13) | day-to-day stock and replenishment management, owned by Manage Inventory Replenishment (CM-1-1-3-7-9) | inventory valuation and accounting, owned by Finance</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Capture Inventory Position | Establish Opening Inventory | Inventory Basis Capture</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node establishes one input of the optimization case, it does not own the underlying business decision or the source data. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. Three inventory nodes are now distinct and must stay that way: this node states the position as a case boundary condition, Plan Finished Goods Inventory (CM-1-1-2-13, approved) sets the plan-period target, and the Inventory cluster (CM-1-1-3-7) owns policy, measurement, reconciliation, and replenishment. The bare taxonomy label “Capture Inventory” is the weakest of the eight and “Capture Inventory Position” is recorded as the preferred alternate label.</t>
+        </is>
+      </c>
+      <c r="U53" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V53" s="5" t="inlineStr">
+        <is>
+          <t>Establish the opening and required closing inventory position bounding the optimization case.</t>
+        </is>
+      </c>
+      <c r="W53" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X53" s="5" t="n"/>
-      <c r="Y53" s="5" t="n"/>
-      <c r="Z53" s="5" t="n"/>
-      <c r="AA53" s="5" t="n"/>
-      <c r="AB53" s="5" t="n"/>
-      <c r="AC53" s="5" t="n"/>
+      <c r="Y53" s="5" t="inlineStr">
+        <is>
+          <t>inventory system of record position | in-transit and committed volumes | minimum operating and unavailable stock levels | plan-period finished-goods inventory target | tankage and segregation constraints</t>
+        </is>
+      </c>
+      <c r="Z53" s="5" t="inlineStr">
+        <is>
+          <t>opening and required closing inventory basis for the optimization case</t>
+        </is>
+      </c>
+      <c r="AA53" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | uses-input: Plan Finished Goods Inventory | informed-by: Measure Inventory | constrained-by: Inventory</t>
+        </is>
+      </c>
+      <c r="AB53" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC53" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD53" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -5456,10 +5828,22 @@
           <t>no meaningful APQC candidate</t>
         </is>
       </c>
-      <c r="U54" s="5" t="n"/>
+      <c r="U54" s="5" t="inlineStr">
+        <is>
+          <t>mixed/needs-review</t>
+        </is>
+      </c>
       <c r="V54" s="5" t="n"/>
       <c r="W54" s="5" t="n"/>
-      <c r="X54" s="5" t="n"/>
+      <c r="X54" s="5" t="inlineStr">
+        <is>
+          <t>Question: Is “Capture Monthly Operating Plan” a process, or does it name the monthly operating plan document itself?
+Context: The seven sibling L5 nodes under Refinery Optimization (CM-1-1-4-7) partition the case basis and its analysis. The monthly operating plan is the output of the optimization cycle, not an input to it, so on a plain reading this node inverts the direction of the sibling set. Its Step 3b APQC candidate was “Plan facility”, scored NONE / NO CANDIDATE, so there is no external signal either way.
+Options: (1) Define it as issuing and registering the approved monthly operating plan as the plan of record handed to Refining for scheduling — a real process, and it closes the optimization cycle; no tree change needed, rename to “Issue Monthly Operating Plan” as preferred label. (2) Define it as loading the current approved operating plan as the starting baseline for the next case — also a real process and a genuine input, but it overlaps the parent scope phrase “current approved operating plan” already covered in the case basis. (3) Classify as not-process, a document rather than an activity, and retire the node; the plan artifact is then represented as the primary_output of CM-1-1-4-7 and CM-1-1-4. (4) Split: keep an issue step here and represent the plan artifact as an output, not a node.
+Evidence: SRC-BJCE-REFPS-001 describes monthly rolling plans as the product of tactical refinery planning, which assigns production targets to process units, and separates planning from scheduling; SRC-SNF-REFPS-001 and SRC-CMU-REFPLAN-001 place the plan as the handover from planning to scheduling. All three support the plan being an output of this cycle, none supports it being captured as an input.
+Recommendation: Option 1. It is the only reading that makes the node a process, leaves the tree unchanged, and gives the optimization cycle an explicit handover step to Refining, which the locked Refining boundary implies but no current node carries. Option 3 is the honest alternative if you would rather not re-point a label. Not defining the row until you decide, because Options 1 and 3 differ on whether the node survives.</t>
+        </is>
+      </c>
       <c r="Y54" s="5" t="n"/>
       <c r="Z54" s="5" t="n"/>
       <c r="AA54" s="5" t="n"/>
@@ -5535,18 +5919,80 @@
           <t>strong APQC candidate but no validator agreed</t>
         </is>
       </c>
-      <c r="U55" s="5" t="n"/>
-      <c r="V55" s="5" t="n"/>
-      <c r="W55" s="5" t="n"/>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Compare alternative production cases by varying crude slate, run rates, product mix, price, or constraint assumptions, and quantify the margin and feasibility consequences of each, so the preferred case and its sensitivities are understood before the plan is approved.</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Covers case-based analysis inside the optimization cycle: defining the scenarios worth testing, running them against the case basis, reading marginal values and binding constraints, quantifying margin and feasibility differences, and documenting the comparison that supports the recommended case. Excludes selecting and approving the production plan, owned by Refinery Planning (CM-1-1-4). Excludes trading and market risk scenarios, owned by Manage And Run Risk Scenarios (CM-1-2-2-3-11). Excludes comparing actual performance to the approved plan, owned by Regional Backcasting (CM-1-1-5) and Distribution Backcasting (CM-1-1-6).</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Define the scenarios and sensitivities worth testing | run alternative cases against the case basis | read marginal values and identify binding constraints | quantify margin, yield, and feasibility differences | document the case comparison supporting the recommendation</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Selecting and approving the production plan, owned by Refinery Planning (CM-1-1-4) | trading and market risk scenarios, owned by Manage And Run Risk Scenarios (CM-1-2-2-3-11) | comparing actuals to the approved plan, owned by Regional Backcasting (CM-1-1-5) and Distribution Backcasting (CM-1-1-6) | investment and strategic configuration studies | optimization model and application administration, owned by Process Excellence &amp; IT</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Perform Case &amp; Sensitivity Analysis | Run Optimization Scenarios | Case Comparison</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18). Read as a case-basis assembly step inside the CM-1-1-4-7 Refinery Optimization run cycle: this node is the analysis step rather than a case-basis input. Sibling “Capture …” nodes were defined together so their boundaries partition the case basis without overlap. Scenario analysis here is forward-looking case comparison within a planning period. It is distinct from backcasting, which is retrospective, and from trading risk scenarios, which test market exposure rather than production alternatives. The APQC candidate “Perform competitive analysis” scored STRONG but is about comparing bidder proposals and was rejected as a false lexical match.</t>
+        </is>
+      </c>
+      <c r="U55" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V55" s="5" t="inlineStr">
+        <is>
+          <t>Quantify and compare production alternatives and their sensitivities to support case selection.</t>
+        </is>
+      </c>
+      <c r="W55" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001 | SRC-BJCE-REFPS-001 | SRC-CMU-REFPLAN-001 | SRC-SNF-REFPS-001</t>
+        </is>
+      </c>
       <c r="X55" s="5" t="n"/>
-      <c r="Y55" s="5" t="n"/>
-      <c r="Z55" s="5" t="n"/>
-      <c r="AA55" s="5" t="n"/>
-      <c r="AB55" s="5" t="n"/>
-      <c r="AC55" s="5" t="n"/>
+      <c r="Y55" s="5" t="inlineStr">
+        <is>
+          <t>assembled case basis of demand, availability, price, constraints, and inventory | base optimization case and solution | candidate scenario definitions | marginal values and binding constraint output</t>
+        </is>
+      </c>
+      <c r="Z55" s="5" t="inlineStr">
+        <is>
+          <t>documented case comparison with margin, feasibility, and sensitivity results</t>
+        </is>
+      </c>
+      <c r="AA55" s="5" t="inlineStr">
+        <is>
+          <t>enables: Refinery Optimization | uses-input: Capture Product Demand Requirements | uses-input: Capture Refinery Level Constraints | precedes: Refinery Planning</t>
+        </is>
+      </c>
+      <c r="AB55" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC55" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD55" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -25316,6 +25762,16 @@
       <c r="N307" t="inlineStr">
         <is>
           <t>Developing a program to promote the objectives, values, products and services of the company to its employees by treating them as potential customers, in order to extend company client base, increase employee engagement or to foster brand advocacy.</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>Covers setting the strategy for communicating brand, offer, and marketing messages to the organization's own employees as an internal audience: audience and channel choice, message and tone direction, and the intended engagement or advocacy outcome. Strategy only. Excludes executing internal communications, owned by Implement Internal Communications (CM-1-3-5-3-9), and excludes campaign-level planning, owned by Marketing Communications Planning (CM-1-3-5-3). Excludes external, media, public, investor, and government communications, which the locked Legal &amp; Corp Comm boundary places outside this branch. Excludes employee relations, terms of employment, and HR policy communication.</t>
+        </is>
+      </c>
+      <c r="T307" t="inlineStr">
+        <is>
+          <t>Batch 02 (2026-09-18), bundled fix. Row was approved in the #29 pre-intake pass with an empty scope_note and has been the single BLOCKING finding of step3c-workbook-validate.py since #30. Only the missing scope_note was added; the approved definition, status, and all other fields are unchanged. Boundaries asserted here are drawn from existing taxonomy siblings and the locked Legal &amp; Corp Comm decision, not from new research. Phase 1 fields remain empty, consistent with this row staying on the PRE_INTAKE_APPROVED allowlist for the later backfill pass.</t>
         </is>
       </c>
       <c r="U307" s="5" t="n"/>
@@ -41563,7 +42019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -42124,6 +42580,100 @@
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SRC-EIA-LFMM-001</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>U.S. Energy Information Administration (DiVita)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Liquid Fuels Market Module refinery LP modeling white paper</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/outlooks/documentation/workshops/pdf/VDiVita%20LFMM%20White%20Paper.pdf</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Government statistical authority</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Refinery LP input categories and model structure; evidence only, not text to copy</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Refinery optimization case basis: assays, availability, prices, specifications, capacities</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SRC-BJCE-REFPS-001</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Brazilian Journal of Chemical Engineering (Moro)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Refinery production planning and scheduling: the refining coordination case</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-18</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.scielo.br/j/bjce/a/GMRKZJGQ5HPqWRPfwKxnWTq/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Peer-reviewed academic</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Planning-versus-scheduling separation and monthly rolling plan evidence; evidence only</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Case-basis inputs, monthly operating plan as planning output, sensitivity analysis</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
Step 3c: review batch 03 — Demand Forecasting
Six rows approved by Hamid 2026-09-19: CM-1-1-1-1 (L4) and its five L5
children. Q1 decided Option A (L4 defined in place as the operational
forecast-production cycle; L3 remains the domain umbrella; no tree
change). Q2 decided Option A (this cluster owns the approved commercial
planning forecast; a binding constraint is recorded for the future
definition of CM-1-2-6-2-3 as Supply And Trading's operational demand
forecasting, per the PTC-002 decide-versus-advise pattern).

Four sources added to the Reference register: EIA STEO, IEA Oil Market
Report, Operations Research Perspectives (Pudasaini 2021), Springer
Lecture Notes in Logistics (Mota, Relvas, Goncalves 2017).

Validation gate: rows=503 approved=34 pending=465 blocked=3 retired=1
blocking=0 questions=0 open_ptc=1. PTC-001 rows untouched.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NsixxJsatanDCYzWQYPc6K
</commit_message>
<xml_diff>
--- a/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
+++ b/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review &amp; authoring'!$A$1:$AD$504</definedName>
@@ -1189,18 +1189,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="5" t="n"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Develop, agree, and publish the recurring product demand forecast that downstream commercial planning runs on — expected demand by product, market, location, and period — by combining a statistical baseline with customer input and market intelligence, and monitor forecast performance so the published forecast remains a reliable planning basis.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Covers the recurring demand-forecast production cycle: preparing forecasting master data and history, developing the statistical baseline, adjusting it with customer input and market intelligence, publishing the approved forecast with its component-level breakdown, and monitoring forecast performance. Its output is the single approved demand forecast consumed by Regional Optimization, Refinery Optimization, and Supply And Trading. Excludes deciding how demand is met — supply, production, inventory, and allocation choices are owned by Regional Optimization (CM-1-1-2); excludes capturing or committing customer orders, owned by Order Management (CM-1-3-7); excludes Supply And Trading's operational refined-product demand forecasting (Forecast Refined Product Demand, CM-1-2-6-2-3), bounded per the batch 03 decision; excludes designing and agreeing the cross-functional forecasting process with sales, owned by Develop &amp; Agree Demand Forecasting Process (CM-1-3-5-1-2).</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Prepare and validate forecasting inputs | develop the statistical baseline forecast | incorporate customer input and market intelligence | publish the approved forecast and component-level forecast plan | monitor forecast accuracy, bias, and adjustment effect</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Supply, production, inventory, and allocation decisions (Regional Optimization, CM-1-1-2) | customer order capture and commitment (Order Management, CM-1-3-7) | trading-side receipt and use of the published forecast (Receive Demand Forecast, CM-1-2-1-1-2) | Supply And Trading operational refined-product demand forecasting (Forecast Refined Product Demand, CM-1-2-6-2-3) | sales forecasting process design (Develop &amp; Agree Demand Forecasting Process, CM-1-3-5-1-2)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Product Demand Forecasting</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). Q1 decision (Hamid, 2026-09-19, Option A): the L4 carries the same label as its L3 parent (CM-1-1-1) and is its only child; authored in place as the operational forecast-production cycle, with the L3 remaining the domain umbrella — no tree change, consistent with the restraint precedent on PTC-001; a later naming pass may disambiguate the duplicate prefLabels. Q2 decision (Hamid, 2026-09-19, Option A): binding constraint on the future definition of CM-1-2-6-2-3 — it must be scoped as Supply And Trading's operational demand forecasting within Refined Product Supply Chain Management and must not claim ownership of the approved commercial planning forecast; same decide-versus-advise pattern as PTC-002. Evidence basis: the planning-cycle forecast (monthly, product/market level; IEA OMR and EIA STEO practice) is distinct from operational network demand forecasting (short-notice, terminal/station level; Mota et al. 2017). APQC 10240 'Evaluate and revise demand forecasting approach' is REVIEW LINK only; approach-governance content sits closest to CM-1-3-5-1-2, not here.</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>Produce and maintain the single approved product demand forecast that downstream commercial planning runs on.</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>SRC-IEA-OMR-001 | SRC-EIA-STEO-001 | SRC-ORP-DPSC-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
-      <c r="Z4" s="5" t="n"/>
-      <c r="AA4" s="5" t="n"/>
-      <c r="AB4" s="5" t="n"/>
-      <c r="AC4" s="5" t="n"/>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>cleansed demand history | customer plans and commitments | market intelligence | product and market master data</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>approved and published demand forecast with component-level forecast plan</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>precedes: Regional Optimization | enables: Capture Product Demand Requirements | enables: Receive Demand Forecast</t>
+        </is>
+      </c>
+      <c r="AB4" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC4" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1268,18 +1330,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U5" s="5" t="n"/>
-      <c r="V5" s="5" t="n"/>
-      <c r="W5" s="5" t="n"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Prepare and validate the reference data and demand history that each forecast cycle depends on — product and market hierarchies, customer and location groupings, units of measure, and the historical demand series cleansed of outliers and one-off distortions — so the statistical baseline is built from accurate, planning-consistent inputs.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Covers per-cycle readiness of forecasting inputs: maintaining forecast-specific reference data, aligning product and market hierarchies to planning definitions, and cleansing demand history for outliers, supply disruptions, and other events that would distort the baseline. Excludes supply-planning reference and parameter data, owned by Maintain Supply Planning Master Data (CM-1-1-2-12); excludes production-scheduling master data, owned by Maintain Production Scheduling Master Data (CM-1-1-7-2-1); excludes customer, price, product, tax, and location master data, owned by Manage Master Data under Order Management (CM-1-3-7-1); excludes enterprise master-data policy and governance, which sit with the Data Governance workstream.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Maintain forecast-specific reference data | align product and market hierarchies to planning definitions | cleanse and adjust demand history for distorting events | validate data readiness for the forecast cycle</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Supply-planning master data (Maintain Supply Planning Master Data, CM-1-1-2-12) | production-scheduling master data (Maintain Production Scheduling Master Data, CM-1-1-7-2-1) | customer, price, product, tax, and location master data (Manage Master Data, CM-1-3-7-1) | enterprise master-data policy and governance (Data Governance workstream) | statistical model development (Develop Statistical Baseline, CM-1-1-1-1-2)</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Forecast Data Preparation</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). Fourth of the four parallel master-data nodes; consolidation under a governed master-data capability is parked for the EPM Data Governance workstream per the decision recorded on CM-1-1-2-12 (2026-09-18) and deliberately not resolved here — the boundary to CM-1-1-2-12 was already established from its approved out_of_scope. APQC 10252 'Maintain master data' is a WEAK distribution-master-data candidate; comparative evidence only.</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>Ensure each forecast cycle starts from validated reference data and cleansed demand history.</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-GLOSS-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X5" s="5" t="n"/>
-      <c r="Y5" s="5" t="n"/>
-      <c r="Z5" s="5" t="n"/>
-      <c r="AA5" s="5" t="n"/>
-      <c r="AB5" s="5" t="n"/>
-      <c r="AC5" s="5" t="n"/>
+      <c r="Y5" s="5" t="inlineStr">
+        <is>
+          <t>raw sales and lifting history | product and market hierarchy definitions | customer and location groupings | recorded demand-distorting events</t>
+        </is>
+      </c>
+      <c r="Z5" s="5" t="inlineStr">
+        <is>
+          <t>validated forecasting dataset and reference data for the cycle</t>
+        </is>
+      </c>
+      <c r="AA5" s="5" t="inlineStr">
+        <is>
+          <t>precedes: Develop Statistical Baseline | enables: Demand Forecasting</t>
+        </is>
+      </c>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC5" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1347,18 +1471,80 @@
           <t>CIRCULAR VALIDATOR (human gate): validator is APQC itself ('Develop baseline demand forecasts', apqc.org benchmarking measures page) validating APQC's own description. Triangulation requires an INDEPENDENT source. No adoption without external agreement.</t>
         </is>
       </c>
-      <c r="U6" s="5" t="n"/>
-      <c r="V6" s="5" t="n"/>
-      <c r="W6" s="5" t="n"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Generate the objective statistical baseline forecast of product demand from cleansed history and demonstrated demand drivers, selecting and tuning forecasting methods by product and market segment before any judgmental input is applied.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Covers producing the unbiased statistical starting point of the forecast cycle: choosing and parameterizing forecasting methods, generating the baseline at the agreed hierarchy levels, and documenting model fit and known limitations. The baseline is deliberately judgment-free — commercial knowledge enters in the adjustment step. Excludes adjusting the forecast with customer input and market intelligence, owned by Adjust Forecast Incorporating Customer Input and Market Intelligence (CM-1-1-1-1-3); excludes publication and disaggregation, owned by Publish Forecast and Generate Component Level Forecast Plan (CM-1-1-1-1-4); excludes measuring forecast performance, owned by Monitor Demand Forecasting Performance and Reporting (CM-1-1-1-1-5).</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Select and tune statistical forecasting methods by segment | generate the baseline forecast at agreed hierarchy levels | apply demonstrated demand drivers | document model fit and limitations</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Judgmental adjustment of the forecast (CM-1-1-1-1-3) | forecast publication and disaggregation (CM-1-1-1-1-4) | forecast performance measurement (CM-1-1-1-1-5) | trading revenue and asset forecasting (Forecasting &amp; Optimization, CM-1-2-1-1)</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Statistical Baseline Forecast | Baseline Forecasting</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). APQC 20043 'Develop baseline forecasts' scored STRONG but was REJECTED at the Step 3b human gate as circular validation (APQC validating APQC); authored independently per that rejection. Driver-based statistical modeling of fuels demand (economic activity, prices, weather) follows the practice documented in EIA STEO product-consumption modules; monthly product-level demand assessment follows IEA OMR practice. 'Baseline' is used in the demand-planning sense — the pre-judgment statistical forecast — not the plan-baseline sense used in backcasting.</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>Produce the objective, judgment-free statistical starting point for the demand forecast.</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-STEO-001 | SRC-IEA-OMR-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X6" s="5" t="n"/>
-      <c r="Y6" s="5" t="n"/>
-      <c r="Z6" s="5" t="n"/>
-      <c r="AA6" s="5" t="n"/>
-      <c r="AB6" s="5" t="n"/>
-      <c r="AC6" s="5" t="n"/>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>validated forecasting dataset | demand driver variables | historical model performance</t>
+        </is>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>statistical baseline forecast by product and market segment</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>follows: Prepare Master Data To Create Demand Forecast | precedes: Adjust Forecast Incorporating Customer Input and Market Intelligence</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC6" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1426,18 +1612,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="5" t="n"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Review and adjust the statistical baseline with demand knowledge the models cannot see — customer plans and commitments, sales and marketing input, and market and competitive intelligence — recording each adjustment and its rationale so the agreed forecast reflects the best available view of demand.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Covers the judgmental overlay and agreement step of the forecast cycle: gathering structured input from customer-facing and market-facing teams, challenging and applying adjustments to the baseline, and recording who changed what and why so performance monitoring can attribute accuracy effects. Excludes producing the statistical baseline itself (CM-1-1-1-1-2); excludes gathering market and customer intelligence as an ongoing capability — this step consumes intelligence, it does not own its production; excludes negotiating or committing the underlying customer volumes, owned by Order Management (CM-1-3-7) and sales.</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Collect structured customer and market input | review and challenge the statistical baseline | apply and document adjustments with rationale | agree the adjusted forecast for publication</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Statistical baseline generation (CM-1-1-1-1-2) | ownership of market and customer intelligence production | customer negotiation and order commitment (Order Management, CM-1-3-7) | publication of the agreed forecast (CM-1-1-1-1-4)</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Consensus Forecast Adjustment | Judgmental Forecast Adjustment</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). Written as the consensus/enrichment step of standard demand-planning practice; the IEA OMR's monthly demand revisions on new market information are the reference pattern for judgment applied over a statistical basis. Adjustments are recorded with rationale specifically so CM-1-1-1-1-5 can measure whether they added accuracy — the adjustment record is part of the process, not an implementation detail. APQC 10106 'Perform customer and market intelligence analysis' is REVIEW LINK; it describes the intelligence capability this step consumes, not this step itself.</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>Turn the statistical baseline into the agreed forecast by applying documented customer and market knowledge.</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr">
+        <is>
+          <t>SRC-IEA-OMR-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X7" s="5" t="n"/>
-      <c r="Y7" s="5" t="n"/>
-      <c r="Z7" s="5" t="n"/>
-      <c r="AA7" s="5" t="n"/>
-      <c r="AB7" s="5" t="n"/>
-      <c r="AC7" s="5" t="n"/>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>statistical baseline forecast | customer plans and commitments | sales and marketing input | market and competitive intelligence</t>
+        </is>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>agreed adjusted forecast with documented adjustment rationale</t>
+        </is>
+      </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>follows: Develop Statistical Baseline | precedes: Publish Forecast and Generate Component Level Forecast Plan</t>
+        </is>
+      </c>
+      <c r="AB7" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC7" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1505,18 +1753,80 @@
           <t>CIRCULAR VALIDATOR (human gate): validator is APQC itself and the cited URL (turnover-rate-manufacturing-personnel) is unrelated to line-level planning; the 'definition' merely restates APQC's own description (agreement 1.0 is self-match). No independent source, no adoption.</t>
         </is>
       </c>
-      <c r="U8" s="5" t="n"/>
-      <c r="V8" s="5" t="n"/>
-      <c r="W8" s="5" t="n"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Approve and publish the agreed demand forecast as the versioned planning basis, and translate it into the component-level forecast plan — the detailed breakdown by product grade or component, location, and period — that downstream planning processes consume.</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Covers the release step of the forecast cycle: final approval, version identification, disaggregation of the agreed forecast to the component level used by planning, and distribution to its consumers. The published version is the fixed reference that both planning and forecast-performance measurement run against. Excludes acting on the forecast — supply, production, inventory, and allocation decisions are owned by Regional Optimization (CM-1-1-2) and Refinery Planning (CM-1-1-4); excludes the consumers' own receipt and case-assembly steps, owned by Receive Demand Forecast (CM-1-2-1-1-2) and Capture Product Demand Requirements (CM-1-1-4-7-1).</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Approve and version the forecast for release | disaggregate to the component-level forecast plan | distribute the published forecast to consuming processes | maintain the published version as the fixed reference for the period</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Supply and allocation decisions (Regional Optimization, CM-1-1-2) | refinery case-basis assembly (Capture Product Demand Requirements, CM-1-1-4-7-1) | trading-side receipt (Receive Demand Forecast, CM-1-2-1-1-2) | forecast adjustment (CM-1-1-1-1-3)</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Forecast Publication | Publish Demand Forecast</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). 'Component level' is read as the detailed disaggregated planning level — product grade or blend component, location, and period — required by the consuming planning processes; the definition states the function without fixing a single technical reading. APQC 10306 'Generate line level plan' scored STRONG but was REJECTED at the Step 3b human gate as circular validation with an unrelated citation; authored independently. The published, versioned forecast is the contemporaneous baseline that CM-1-1-1-1-5 measures against — consistent with the locked backcasting discipline.</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>Release one versioned, detailed demand forecast that all downstream planning consumes.</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-STEO-001 | SRC-ORP-DPSC-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X8" s="5" t="n"/>
-      <c r="Y8" s="5" t="n"/>
-      <c r="Z8" s="5" t="n"/>
-      <c r="AA8" s="5" t="n"/>
-      <c r="AB8" s="5" t="n"/>
-      <c r="AC8" s="5" t="n"/>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>agreed adjusted forecast | product component and grade structures | planning calendar</t>
+        </is>
+      </c>
+      <c r="Z8" s="5" t="inlineStr">
+        <is>
+          <t>published versioned demand forecast and component-level forecast plan</t>
+        </is>
+      </c>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>follows: Adjust Forecast Incorporating Customer Input and Market Intelligence | precedes: Regional Optimization | enables: Capture Product Demand Requirements | enables: Receive Demand Forecast</t>
+        </is>
+      </c>
+      <c r="AB8" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC8" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1584,18 +1894,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U9" s="5" t="n"/>
-      <c r="V9" s="5" t="n"/>
-      <c r="W9" s="5" t="n"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Measure and report how well published demand forecasts predicted actual demand — tracking accuracy, bias, and the effect of adjustments at agreed levels and lags — and feed the findings back into forecasting methods and adjustment behavior.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Covers recurring forecast-performance measurement and reporting: comparing actual demand with the forecast as published for that period, analyzing error and bias by segment and lag, evaluating whether judgmental adjustments improved accuracy, reporting results, and recommending method and process improvements. Actuals are compared with the contemporaneously published forecast version, not a later revision. Excludes explaining supply-plan versus actual outcomes, owned by Regional Backcasting (CM-1-1-5) and Distribution Backcasting (CM-1-1-6); excludes agreeing the cross-functional forecasting process design with sales, owned by Develop &amp; Agree Demand Forecasting Process (CM-1-3-5-1-2).</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Compare actual demand with the published forecast version | analyze forecast error and bias by segment and lag | evaluate the accuracy effect of judgmental adjustments | report performance and recommend improvements</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Plan-versus-actual supply and distribution variance analysis (Regional Backcasting, CM-1-1-5; Distribution Backcasting, CM-1-1-6) | forecasting process design and agreement (Develop &amp; Agree Demand Forecasting Process, CM-1-3-5-1-2) | making the forecast adjustments themselves (CM-1-1-1-1-3)</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Forecast Accuracy Monitoring | Forecast Performance Measurement</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). Measures the forecast against actual demand using the as-published version as the fixed comparison basis — the same contemporaneous-baseline discipline locked for Regional and Distribution Backcasting, applied to the demand side. EIA's published STEO forecast-accuracy evaluations are the reference practice for measuring product-demand forecasts against realized data. Specific accuracy metrics and thresholds are deliberately not named; they belong to the KPI workstream, not the process definition. APQC 16574 'Monitor and report performance' is a WEAK marketing-channel candidate; comparative evidence only.</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>Establish whether published forecasts are getting more or less reliable, and why, so the forecasting cycle improves.</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-STEO-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X9" s="5" t="n"/>
-      <c r="Y9" s="5" t="n"/>
-      <c r="Z9" s="5" t="n"/>
-      <c r="AA9" s="5" t="n"/>
-      <c r="AB9" s="5" t="n"/>
-      <c r="AC9" s="5" t="n"/>
+      <c r="Y9" s="5" t="inlineStr">
+        <is>
+          <t>published forecast versions | actual demand history | adjustment records with rationale</t>
+        </is>
+      </c>
+      <c r="Z9" s="5" t="inlineStr">
+        <is>
+          <t>forecast performance report with improvement recommendations</t>
+        </is>
+      </c>
+      <c r="AA9" s="5" t="inlineStr">
+        <is>
+          <t>follows: Publish Forecast and Generate Component Level Forecast Plan | uses-input: Adjust Forecast Incorporating Customer Input and Market Intelligence | enables: Demand Forecasting</t>
+        </is>
+      </c>
+      <c r="AB9" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC9" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -42081,7 +42453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -42130,6 +42502,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
@@ -42736,6 +43109,194 @@
         </is>
       </c>
       <c r="I19" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SRC-EIA-STEO-001</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>U.S. Energy Information Administration</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Short-Term Energy Outlook and model documentation (petroleum product consumption modules)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/outlooks/steo/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Government statistical authority</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Petroleum-product demand forecasting practice and driver-based modeling; evidence only, not text to copy</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Statistical modeling of product demand by fuel, region, and driver variables (economic activity, prices, weather); published forecast-accuracy evaluation</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SRC-IEA-OMR-001</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>International Energy Agency</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Oil Market Report (monthly series)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.iea.org/reports/oil-market-report</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Intergovernmental energy authority</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Product-level oil demand assessment and forecast practice; evidence only, not text to copy</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Monthly demand-by-product-and-region assessment cycle and revision practice</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SRC-ORP-DPSC-001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Operations Research Perspectives (Pudasaini)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Integrated planning of downstream petroleum supply chain: a multi-objective stochastic approach</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Vol. 8, 2021; accessed 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S2214716021000129</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Peer-reviewed academic</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Downstream planning structure and demand as planning input; evidence only</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Demand as the driving input of downstream supply and distribution network planning</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SRC-LNL-T2S-001</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Springer Lecture Notes in Logistics (Mota, Relvas, Goncalves)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Downstream Oil Products Distribution Planning: A Portuguese Case Study</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2017; accessed 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-319-42421-7_3</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Peer-reviewed academic</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Secondary-distribution planning and short-term network demand; evidence only</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Operational terminal/station-level demand versus the planning-cycle forecast (batch 03 Q2 boundary evidence)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
Step 3c: review batch 03 — Demand Forecasting (#37)
Six rows approved by Hamid 2026-09-19: CM-1-1-1-1 (L4) and its five L5
children. Q1 decided Option A (L4 defined in place as the operational
forecast-production cycle; L3 remains the domain umbrella; no tree
change). Q2 decided Option A (this cluster owns the approved commercial
planning forecast; a binding constraint is recorded for the future
definition of CM-1-2-6-2-3 as Supply And Trading's operational demand
forecasting, per the PTC-002 decide-versus-advise pattern).

Four sources added to the Reference register: EIA STEO, IEA Oil Market
Report, Operations Research Perspectives (Pudasaini 2021), Springer
Lecture Notes in Logistics (Mota, Relvas, Goncalves 2017).

Validation gate: rows=503 approved=34 pending=465 blocked=3 retired=1
blocking=0 questions=0 open_ptc=1. PTC-001 rows untouched.


Claude-Session: https://claude.ai/code/session_01NsixxJsatanDCYzWQYPc6K

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
+++ b/business_architecture/ontology/build/output/step3c-definition-authoring-workbook.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Start Here — Decisions &amp; Phases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Review &amp; authoring" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Column guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Controlled vocabularies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reference register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="External mappings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review &amp; authoring'!$A$1:$AD$504</definedName>
@@ -1189,18 +1189,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="5" t="n"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Develop, agree, and publish the recurring product demand forecast that downstream commercial planning runs on — expected demand by product, market, location, and period — by combining a statistical baseline with customer input and market intelligence, and monitor forecast performance so the published forecast remains a reliable planning basis.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Covers the recurring demand-forecast production cycle: preparing forecasting master data and history, developing the statistical baseline, adjusting it with customer input and market intelligence, publishing the approved forecast with its component-level breakdown, and monitoring forecast performance. Its output is the single approved demand forecast consumed by Regional Optimization, Refinery Optimization, and Supply And Trading. Excludes deciding how demand is met — supply, production, inventory, and allocation choices are owned by Regional Optimization (CM-1-1-2); excludes capturing or committing customer orders, owned by Order Management (CM-1-3-7); excludes Supply And Trading's operational refined-product demand forecasting (Forecast Refined Product Demand, CM-1-2-6-2-3), bounded per the batch 03 decision; excludes designing and agreeing the cross-functional forecasting process with sales, owned by Develop &amp; Agree Demand Forecasting Process (CM-1-3-5-1-2).</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Prepare and validate forecasting inputs | develop the statistical baseline forecast | incorporate customer input and market intelligence | publish the approved forecast and component-level forecast plan | monitor forecast accuracy, bias, and adjustment effect</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Supply, production, inventory, and allocation decisions (Regional Optimization, CM-1-1-2) | customer order capture and commitment (Order Management, CM-1-3-7) | trading-side receipt and use of the published forecast (Receive Demand Forecast, CM-1-2-1-1-2) | Supply And Trading operational refined-product demand forecasting (Forecast Refined Product Demand, CM-1-2-6-2-3) | sales forecasting process design (Develop &amp; Agree Demand Forecasting Process, CM-1-3-5-1-2)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Product Demand Forecasting</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). Q1 decision (Hamid, 2026-09-19, Option A): the L4 carries the same label as its L3 parent (CM-1-1-1) and is its only child; authored in place as the operational forecast-production cycle, with the L3 remaining the domain umbrella — no tree change, consistent with the restraint precedent on PTC-001; a later naming pass may disambiguate the duplicate prefLabels. Q2 decision (Hamid, 2026-09-19, Option A): binding constraint on the future definition of CM-1-2-6-2-3 — it must be scoped as Supply And Trading's operational demand forecasting within Refined Product Supply Chain Management and must not claim ownership of the approved commercial planning forecast; same decide-versus-advise pattern as PTC-002. Evidence basis: the planning-cycle forecast (monthly, product/market level; IEA OMR and EIA STEO practice) is distinct from operational network demand forecasting (short-notice, terminal/station level; Mota et al. 2017). APQC 10240 'Evaluate and revise demand forecasting approach' is REVIEW LINK only; approach-governance content sits closest to CM-1-3-5-1-2, not here.</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>Produce and maintain the single approved product demand forecast that downstream commercial planning runs on.</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>SRC-IEA-OMR-001 | SRC-EIA-STEO-001 | SRC-ORP-DPSC-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
-      <c r="Z4" s="5" t="n"/>
-      <c r="AA4" s="5" t="n"/>
-      <c r="AB4" s="5" t="n"/>
-      <c r="AC4" s="5" t="n"/>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>cleansed demand history | customer plans and commitments | market intelligence | product and market master data</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>approved and published demand forecast with component-level forecast plan</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>precedes: Regional Optimization | enables: Capture Product Demand Requirements | enables: Receive Demand Forecast</t>
+        </is>
+      </c>
+      <c r="AB4" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC4" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1268,18 +1330,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U5" s="5" t="n"/>
-      <c r="V5" s="5" t="n"/>
-      <c r="W5" s="5" t="n"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Prepare and validate the reference data and demand history that each forecast cycle depends on — product and market hierarchies, customer and location groupings, units of measure, and the historical demand series cleansed of outliers and one-off distortions — so the statistical baseline is built from accurate, planning-consistent inputs.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Covers per-cycle readiness of forecasting inputs: maintaining forecast-specific reference data, aligning product and market hierarchies to planning definitions, and cleansing demand history for outliers, supply disruptions, and other events that would distort the baseline. Excludes supply-planning reference and parameter data, owned by Maintain Supply Planning Master Data (CM-1-1-2-12); excludes production-scheduling master data, owned by Maintain Production Scheduling Master Data (CM-1-1-7-2-1); excludes customer, price, product, tax, and location master data, owned by Manage Master Data under Order Management (CM-1-3-7-1); excludes enterprise master-data policy and governance, which sit with the Data Governance workstream.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Maintain forecast-specific reference data | align product and market hierarchies to planning definitions | cleanse and adjust demand history for distorting events | validate data readiness for the forecast cycle</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Supply-planning master data (Maintain Supply Planning Master Data, CM-1-1-2-12) | production-scheduling master data (Maintain Production Scheduling Master Data, CM-1-1-7-2-1) | customer, price, product, tax, and location master data (Manage Master Data, CM-1-3-7-1) | enterprise master-data policy and governance (Data Governance workstream) | statistical model development (Develop Statistical Baseline, CM-1-1-1-1-2)</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Forecast Data Preparation</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). Fourth of the four parallel master-data nodes; consolidation under a governed master-data capability is parked for the EPM Data Governance workstream per the decision recorded on CM-1-1-2-12 (2026-09-18) and deliberately not resolved here — the boundary to CM-1-1-2-12 was already established from its approved out_of_scope. APQC 10252 'Maintain master data' is a WEAK distribution-master-data candidate; comparative evidence only.</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>Ensure each forecast cycle starts from validated reference data and cleansed demand history.</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-GLOSS-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X5" s="5" t="n"/>
-      <c r="Y5" s="5" t="n"/>
-      <c r="Z5" s="5" t="n"/>
-      <c r="AA5" s="5" t="n"/>
-      <c r="AB5" s="5" t="n"/>
-      <c r="AC5" s="5" t="n"/>
+      <c r="Y5" s="5" t="inlineStr">
+        <is>
+          <t>raw sales and lifting history | product and market hierarchy definitions | customer and location groupings | recorded demand-distorting events</t>
+        </is>
+      </c>
+      <c r="Z5" s="5" t="inlineStr">
+        <is>
+          <t>validated forecasting dataset and reference data for the cycle</t>
+        </is>
+      </c>
+      <c r="AA5" s="5" t="inlineStr">
+        <is>
+          <t>precedes: Develop Statistical Baseline | enables: Demand Forecasting</t>
+        </is>
+      </c>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC5" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1347,18 +1471,80 @@
           <t>CIRCULAR VALIDATOR (human gate): validator is APQC itself ('Develop baseline demand forecasts', apqc.org benchmarking measures page) validating APQC's own description. Triangulation requires an INDEPENDENT source. No adoption without external agreement.</t>
         </is>
       </c>
-      <c r="U6" s="5" t="n"/>
-      <c r="V6" s="5" t="n"/>
-      <c r="W6" s="5" t="n"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Generate the objective statistical baseline forecast of product demand from cleansed history and demonstrated demand drivers, selecting and tuning forecasting methods by product and market segment before any judgmental input is applied.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Covers producing the unbiased statistical starting point of the forecast cycle: choosing and parameterizing forecasting methods, generating the baseline at the agreed hierarchy levels, and documenting model fit and known limitations. The baseline is deliberately judgment-free — commercial knowledge enters in the adjustment step. Excludes adjusting the forecast with customer input and market intelligence, owned by Adjust Forecast Incorporating Customer Input and Market Intelligence (CM-1-1-1-1-3); excludes publication and disaggregation, owned by Publish Forecast and Generate Component Level Forecast Plan (CM-1-1-1-1-4); excludes measuring forecast performance, owned by Monitor Demand Forecasting Performance and Reporting (CM-1-1-1-1-5).</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Select and tune statistical forecasting methods by segment | generate the baseline forecast at agreed hierarchy levels | apply demonstrated demand drivers | document model fit and limitations</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Judgmental adjustment of the forecast (CM-1-1-1-1-3) | forecast publication and disaggregation (CM-1-1-1-1-4) | forecast performance measurement (CM-1-1-1-1-5) | trading revenue and asset forecasting (Forecasting &amp; Optimization, CM-1-2-1-1)</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Statistical Baseline Forecast | Baseline Forecasting</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). APQC 20043 'Develop baseline forecasts' scored STRONG but was REJECTED at the Step 3b human gate as circular validation (APQC validating APQC); authored independently per that rejection. Driver-based statistical modeling of fuels demand (economic activity, prices, weather) follows the practice documented in EIA STEO product-consumption modules; monthly product-level demand assessment follows IEA OMR practice. 'Baseline' is used in the demand-planning sense — the pre-judgment statistical forecast — not the plan-baseline sense used in backcasting.</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>Produce the objective, judgment-free statistical starting point for the demand forecast.</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-STEO-001 | SRC-IEA-OMR-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X6" s="5" t="n"/>
-      <c r="Y6" s="5" t="n"/>
-      <c r="Z6" s="5" t="n"/>
-      <c r="AA6" s="5" t="n"/>
-      <c r="AB6" s="5" t="n"/>
-      <c r="AC6" s="5" t="n"/>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>validated forecasting dataset | demand driver variables | historical model performance</t>
+        </is>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>statistical baseline forecast by product and market segment</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>follows: Prepare Master Data To Create Demand Forecast | precedes: Adjust Forecast Incorporating Customer Input and Market Intelligence</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC6" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1426,18 +1612,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="5" t="n"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Review and adjust the statistical baseline with demand knowledge the models cannot see — customer plans and commitments, sales and marketing input, and market and competitive intelligence — recording each adjustment and its rationale so the agreed forecast reflects the best available view of demand.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Covers the judgmental overlay and agreement step of the forecast cycle: gathering structured input from customer-facing and market-facing teams, challenging and applying adjustments to the baseline, and recording who changed what and why so performance monitoring can attribute accuracy effects. Excludes producing the statistical baseline itself (CM-1-1-1-1-2); excludes gathering market and customer intelligence as an ongoing capability — this step consumes intelligence, it does not own its production; excludes negotiating or committing the underlying customer volumes, owned by Order Management (CM-1-3-7) and sales.</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Collect structured customer and market input | review and challenge the statistical baseline | apply and document adjustments with rationale | agree the adjusted forecast for publication</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Statistical baseline generation (CM-1-1-1-1-2) | ownership of market and customer intelligence production | customer negotiation and order commitment (Order Management, CM-1-3-7) | publication of the agreed forecast (CM-1-1-1-1-4)</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Consensus Forecast Adjustment | Judgmental Forecast Adjustment</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). Written as the consensus/enrichment step of standard demand-planning practice; the IEA OMR's monthly demand revisions on new market information are the reference pattern for judgment applied over a statistical basis. Adjustments are recorded with rationale specifically so CM-1-1-1-1-5 can measure whether they added accuracy — the adjustment record is part of the process, not an implementation detail. APQC 10106 'Perform customer and market intelligence analysis' is REVIEW LINK; it describes the intelligence capability this step consumes, not this step itself.</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>Turn the statistical baseline into the agreed forecast by applying documented customer and market knowledge.</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr">
+        <is>
+          <t>SRC-IEA-OMR-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X7" s="5" t="n"/>
-      <c r="Y7" s="5" t="n"/>
-      <c r="Z7" s="5" t="n"/>
-      <c r="AA7" s="5" t="n"/>
-      <c r="AB7" s="5" t="n"/>
-      <c r="AC7" s="5" t="n"/>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>statistical baseline forecast | customer plans and commitments | sales and marketing input | market and competitive intelligence</t>
+        </is>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>agreed adjusted forecast with documented adjustment rationale</t>
+        </is>
+      </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>follows: Develop Statistical Baseline | precedes: Publish Forecast and Generate Component Level Forecast Plan</t>
+        </is>
+      </c>
+      <c r="AB7" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC7" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1505,18 +1753,80 @@
           <t>CIRCULAR VALIDATOR (human gate): validator is APQC itself and the cited URL (turnover-rate-manufacturing-personnel) is unrelated to line-level planning; the 'definition' merely restates APQC's own description (agreement 1.0 is self-match). No independent source, no adoption.</t>
         </is>
       </c>
-      <c r="U8" s="5" t="n"/>
-      <c r="V8" s="5" t="n"/>
-      <c r="W8" s="5" t="n"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Approve and publish the agreed demand forecast as the versioned planning basis, and translate it into the component-level forecast plan — the detailed breakdown by product grade or component, location, and period — that downstream planning processes consume.</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Covers the release step of the forecast cycle: final approval, version identification, disaggregation of the agreed forecast to the component level used by planning, and distribution to its consumers. The published version is the fixed reference that both planning and forecast-performance measurement run against. Excludes acting on the forecast — supply, production, inventory, and allocation decisions are owned by Regional Optimization (CM-1-1-2) and Refinery Planning (CM-1-1-4); excludes the consumers' own receipt and case-assembly steps, owned by Receive Demand Forecast (CM-1-2-1-1-2) and Capture Product Demand Requirements (CM-1-1-4-7-1).</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Approve and version the forecast for release | disaggregate to the component-level forecast plan | distribute the published forecast to consuming processes | maintain the published version as the fixed reference for the period</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Supply and allocation decisions (Regional Optimization, CM-1-1-2) | refinery case-basis assembly (Capture Product Demand Requirements, CM-1-1-4-7-1) | trading-side receipt (Receive Demand Forecast, CM-1-2-1-1-2) | forecast adjustment (CM-1-1-1-1-3)</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Forecast Publication | Publish Demand Forecast</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). 'Component level' is read as the detailed disaggregated planning level — product grade or blend component, location, and period — required by the consuming planning processes; the definition states the function without fixing a single technical reading. APQC 10306 'Generate line level plan' scored STRONG but was REJECTED at the Step 3b human gate as circular validation with an unrelated citation; authored independently. The published, versioned forecast is the contemporaneous baseline that CM-1-1-1-1-5 measures against — consistent with the locked backcasting discipline.</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>Release one versioned, detailed demand forecast that all downstream planning consumes.</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-STEO-001 | SRC-ORP-DPSC-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X8" s="5" t="n"/>
-      <c r="Y8" s="5" t="n"/>
-      <c r="Z8" s="5" t="n"/>
-      <c r="AA8" s="5" t="n"/>
-      <c r="AB8" s="5" t="n"/>
-      <c r="AC8" s="5" t="n"/>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>agreed adjusted forecast | product component and grade structures | planning calendar</t>
+        </is>
+      </c>
+      <c r="Z8" s="5" t="inlineStr">
+        <is>
+          <t>published versioned demand forecast and component-level forecast plan</t>
+        </is>
+      </c>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>follows: Adjust Forecast Incorporating Customer Input and Market Intelligence | precedes: Regional Optimization | enables: Capture Product Demand Requirements | enables: Receive Demand Forecast</t>
+        </is>
+      </c>
+      <c r="AB8" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC8" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -1584,18 +1894,80 @@
           <t>weak APQC candidate; manual review needed</t>
         </is>
       </c>
-      <c r="U9" s="5" t="n"/>
-      <c r="V9" s="5" t="n"/>
-      <c r="W9" s="5" t="n"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Measure and report how well published demand forecasts predicted actual demand — tracking accuracy, bias, and the effect of adjustments at agreed levels and lags — and feed the findings back into forecasting methods and adjustment behavior.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Covers recurring forecast-performance measurement and reporting: comparing actual demand with the forecast as published for that period, analyzing error and bias by segment and lag, evaluating whether judgmental adjustments improved accuracy, reporting results, and recommending method and process improvements. Actuals are compared with the contemporaneously published forecast version, not a later revision. Excludes explaining supply-plan versus actual outcomes, owned by Regional Backcasting (CM-1-1-5) and Distribution Backcasting (CM-1-1-6); excludes agreeing the cross-functional forecasting process design with sales, owned by Develop &amp; Agree Demand Forecasting Process (CM-1-3-5-1-2).</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Compare actual demand with the published forecast version | analyze forecast error and bias by segment and lag | evaluate the accuracy effect of judgmental adjustments | report performance and recommend improvements</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Plan-versus-actual supply and distribution variance analysis (Regional Backcasting, CM-1-1-5; Distribution Backcasting, CM-1-1-6) | forecasting process design and agreement (Develop &amp; Agree Demand Forecasting Process, CM-1-3-5-1-2) | making the forecast adjustments themselves (CM-1-1-1-1-3)</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Forecast Accuracy Monitoring | Forecast Performance Measurement</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Batch 03 (2026-09-19). Measures the forecast against actual demand using the as-published version as the fixed comparison basis — the same contemporaneous-baseline discipline locked for Regional and Distribution Backcasting, applied to the demand side. EIA's published STEO forecast-accuracy evaluations are the reference practice for measuring product-demand forecasts against realized data. Specific accuracy metrics and thresholds are deliberately not named; they belong to the KPI workstream, not the process definition. APQC 16574 'Monitor and report performance' is a WEAK marketing-channel candidate; comparative evidence only.</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>Establish whether published forecasts are getting more or less reliable, and why, so the forecasting cycle improves.</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="inlineStr">
+        <is>
+          <t>SRC-EIA-STEO-001 | SRC-ASCM-CSCP-001</t>
+        </is>
+      </c>
       <c r="X9" s="5" t="n"/>
-      <c r="Y9" s="5" t="n"/>
-      <c r="Z9" s="5" t="n"/>
-      <c r="AA9" s="5" t="n"/>
-      <c r="AB9" s="5" t="n"/>
-      <c r="AC9" s="5" t="n"/>
+      <c r="Y9" s="5" t="inlineStr">
+        <is>
+          <t>published forecast versions | actual demand history | adjustment records with rationale</t>
+        </is>
+      </c>
+      <c r="Z9" s="5" t="inlineStr">
+        <is>
+          <t>forecast performance report with improvement recommendations</t>
+        </is>
+      </c>
+      <c r="AA9" s="5" t="inlineStr">
+        <is>
+          <t>follows: Publish Forecast and Generate Component Level Forecast Plan | uses-input: Adjust Forecast Incorporating Customer Input and Market Intelligence | enables: Demand Forecasting</t>
+        </is>
+      </c>
+      <c r="AB9" s="5" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="AC9" s="5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -42081,7 +42453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -42130,6 +42502,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
@@ -42736,6 +43109,194 @@
         </is>
       </c>
       <c r="I19" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SRC-EIA-STEO-001</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>U.S. Energy Information Administration</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Short-Term Energy Outlook and model documentation (petroleum product consumption modules)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/outlooks/steo/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Government statistical authority</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Petroleum-product demand forecasting practice and driver-based modeling; evidence only, not text to copy</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Statistical modeling of product demand by fuel, region, and driver variables (economic activity, prices, weather); published forecast-accuracy evaluation</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SRC-IEA-OMR-001</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>International Energy Agency</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Oil Market Report (monthly series)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Accessed 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.iea.org/reports/oil-market-report</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Intergovernmental energy authority</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Product-level oil demand assessment and forecast practice; evidence only, not text to copy</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Monthly demand-by-product-and-region assessment cycle and revision practice</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SRC-ORP-DPSC-001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Operations Research Perspectives (Pudasaini)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Integrated planning of downstream petroleum supply chain: a multi-objective stochastic approach</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Vol. 8, 2021; accessed 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S2214716021000129</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Peer-reviewed academic</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Downstream planning structure and demand as planning input; evidence only</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Demand as the driving input of downstream supply and distribution network planning</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SRC-LNL-T2S-001</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Springer Lecture Notes in Logistics (Mota, Relvas, Goncalves)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Downstream Oil Products Distribution Planning: A Portuguese Case Study</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2017; accessed 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/978-3-319-42421-7_3</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Peer-reviewed academic</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Secondary-distribution planning and short-term network demand; evidence only</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Operational terminal/station-level demand versus the planning-cycle forecast (batch 03 Q2 boundary evidence)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>